<commit_message>
feat: Implement backup management feature
- Added backup management screen with functionality to trigger manual backups, view backup history, and manage automated backup settings.
- Introduced BackupService for handling backup-related API interactions.
- Updated localization files for English and French to include new backup management strings.
- Created models for BackupSettings and BackupRecord to manage backup data.
- Enhanced user roles to include permission for managing backups.
- Updated main navigation to include backup management.
- Added API endpoint for backups in the configuration.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -528,6 +528,40 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Gestion des Sauvegardes</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Page d'administration pour déclencher, automatiser, et télécharger les sauvegardes de la base de données hospital.db avec rappel de stockage externe.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Tables backup_settings + backup_history dans db-service. Route /api/admin/backups. Permission manageBackups (admin). Flutter : BackupManagementScreen + BackupService Singleton.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Enhance issue detail view with enriched data
- Implemented a new endpoint to retrieve detailed issue information including related equipment, audit logs, and maintenance records.
- Added localization strings for issue detail sections in English and French.
- Created a new model for issue details, including audit entries and maintenance records.
- Developed a dedicated screen for displaying issue details with structured sections for context, failure, intervention, maintenance history, and timeline.
- Updated the issue tracking screen to navigate to the new issue detail screen instead of using a dialog.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -562,6 +562,40 @@
         </is>
       </c>
     </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Page Détail Incident (GMAO)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Remplacement du pop-up par une page complète affichant le cycle de vie, la cause racine, les pièces et l'historique de l'incident.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Backend enrichi (GET /api/issues/:id) avec équipement, audit trail et maintenance. Écran IssueDetailScreen avec 5 sections GMAO et timeline verticale. flutter analyze : 0 erreur. npm test : 32/32.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Add preventive maintenance protocols and criticality classification
- Introduced new localization strings for macro-categories, sub-categories, and criticality levels in English and French.
- Updated the `Equipment` model to include fields for sub-category, macro-category, warranty end date, and criticality.
- Created a new `PmProtocol` model for managing preventive maintenance protocols associated with equipment types.
- Enhanced the `IssueFormScreen` to utilize macro-categories for filtering biomedical and IT equipment.
- Added warranty alert logic to the `Equipment` model to track warranty expiration.
- Updated localization files and localization classes to support new strings and methods.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -596,6 +596,74 @@
         </is>
       </c>
     </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Hiérarchie GMAO : macro-catégories &amp; sous-catégories</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Ajout des tables equipment_macro_categories (Biomedical/Infrastructure/IT), equipment_subcategories (~626 entrées migrées), pm_protocols avec seed pour 8 types biomédicaux. Colonnes subcategory_id, macro_category_id, warranty_end_date, criticality sur equipment. Routes /api/categories et /api/pm-protocols. Modèles Flutter mis à jour (Equipment + PmProtocol). Filtrage IssueFormScreen basculé de category-text vers macroCategory.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>32 tests Jest passent. flutter analyze --no-fatal-infos : 46 info préexistants, 0 erreur. Migration DB 100% idempotente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>GMAO Phase 2 - Hiérarchie équipements &amp; protocoles PM</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Refonte classification : macro-catégories (Biomedical/Infrastructure/IT), sous-catégories migrées depuis ~626 equipment_categories, table pm_protocols avec checklist JSON, champs criticality (A/B/C) et warranty_end_date sur equipment. CRUD backend + modèles Flutter mis à jour.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>8 protocoles PM biomédicaux seedés. flutter analyze : 46 infos pré-existantes, 0 erreur. npm test : 32 passed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Enhance equipment detail screen with criticality and warranty information
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -664,6 +664,36 @@
         </is>
       </c>
     </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Amélioration EquipmentDetailScreen</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Refonte de la vue détail équipement : ajout criticité (A/B/C colorée), garantie avec badge d'état, macro-catégorie, sous-catégorie, et incidents cliquables naviguant vers IssueDetailScreen</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add system status messages and recent account feature to login screen
- Updated English and French localization files to include new system status messages, alert banners, and recent session titles.
- Enhanced `AppLocalizations` classes to support new strings for system status and alerts.
- Modified `login_screen.dart` to display system health status, recent accounts, and improved UI for alerts and buttons.
- Added functionality to fetch and display system health status with real-time updates.
- Improved layout and organization of the login screen for better user experience.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -694,6 +694,40 @@
       <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr"/>
     </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Refonte écran login GMAO</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Séparation claire des 3 modes (connexion/inscription/reset), suppression du champ rôle à l'inscription, sécurisation des boutons DEV via kDebugMode, bannière d'alerte service, footer statut système, bouton 'Mot de passe oublié' proéminent, section comptes récents, 9 nouvelles clés i18n FR+EN.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Tous les flux i18n générés. flutter analyze --no-fatal-infos OK. Aucune régression détectée.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Refactor login screen layout for responsive design and remove recent accounts section
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -728,6 +728,40 @@
         </is>
       </c>
     </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Login - layout responsive bureau/mobile</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Mise en page 2 colonnes sur bureau (≥800px, logo gauche, formulaire droit, pas de scroll global), layout mobile scroll sans comptes récents, statut système coin bas-droit, bouton langue affiche la langue courante (FR/EN).</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>flutter analyze --no-fatal-infos OK. Breakpoint 800px cohérent avec le reste de l'app.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Add global dashboard with KPIs and quick access features to home hub screen
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -762,6 +762,40 @@
         </is>
       </c>
     </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Redirection intelligente et Hub KPIs</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Redirection post-login basée sur le rôle (techniciens → IssueTracking direct). HomeHubScreen transformé en tableau de bord global GMAO avec 3 tuiles KPI dynamiques (incidents critiques/urgents, alertes stock, équipements hors service), FAB urgence 'Signaler un incident' et badges d'alerte sur les cartes modules.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Testé flutter analyze --no-fatal-infos. i18n FR+EN ajoutée (12 nouvelles clés). Visibilité RBAC des cartes modules respectée.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Enhance dashboard functionality with data freshness indicators and priority incident metrics
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -796,6 +796,40 @@
         </is>
       </c>
     </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Refonte Dashboard GMAO</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Refonte du tableau de bord : 5e StatCard PM en retard, tri incidents par urgence décroissante, alertes incidents critiques &gt;24h, indicateurs opérationnels technicien/superviseur, panel latéral desktop équipements critiques HS, indicateur de fraîcheur des données.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>13 nouvelles clés i18n (FR+EN). Layout RBAC : vue simplifiée pour hospitalStaff, vue étendue pour techniciens/superviseurs/admins. 3e colonne desktop technicien. flutter analyze --no-fatal-infos OK.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Add CSV export functionality with platform-specific implementations
- Implemented a selector for CSV export based on the platform in `csv_export.dart`.
- Created a stub implementation in `csv_export_stub.dart` that returns false for non-web platforms.
- Developed a web-specific implementation in `csv_export_web.dart` that triggers CSV downloads in the browser.
- Updated the `suivi_verifications.xlsx` file.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -830,6 +830,40 @@
         </is>
       </c>
     </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Refonte EquipmentListScreen</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Virtualisation SliverList, RBAC colonnes par rôle, formulaire Stepper 3 étapes, filtre PM, bouton Planifier PM, export CSV liste filtrée</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Correction bonus : clés ARB dashboard manquantes du commit précédent. flutter analyze --no-fatal-infos : EXIT 0.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Add Equipment QR Dialog and Staff View
- Implemented EquipmentQrDialog to display equipment ID as a QR code and allow copying to clipboard.
- Created EquipmentStaffView for hospital staff, showcasing critical alerts, equipment status, active issues, and contact information.
- Introduced KanbanBoard for issue management with columns for different statuses.
- Added ReportKpiSection to display KPIs including MTTR and PM compliance.
- Updated macOS plugin registration to include mobile_scanner.
- Updated pubspec.yaml and pubspec.lock to include new dependencies: mobile_scanner and fl_chart.
- Updated verification spreadsheet.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -864,6 +864,240 @@
         </is>
       </c>
     </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-012</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Refonte EquipmentDetailScreen</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Décomposition de l'écran monolithique (925 lignes) en 8 sous-widgets, navigation par onglets, vue RBAC hospitalStaff simplifiée, bannière critique, QR Code, MTTR, bouton PM, double confirmation suppression</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>8 nouveaux fichiers dans lib/widgets/equipment/. ARB : 34 nouvelles clés FR+EN. flutter analyze --no-fatal-infos : 0 erreur/warning dans les nouveaux fichiers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Refonte IssueFormScreen — UX &amp; GMAO</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Garde-fou changement d'onglet, scanner QR biomédical, aperçu photo plein écran, switch disponibilité équipement, modale succès avec ticket ID et SLA par urgence.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>mobile_scanner ^6.0.0 ajouté. Sur web : fallback dialog saisie manuelle ID. SLA : Critique=2h, Urgent=12h, Moyen=48h, Faible=1sem. flutter gen-l10n régénéré.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-014</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Refonte IssueTrackingScreen GMAO</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Ajout recherche globale, filtres avancés (statut/urgence/période/groupe), tri urgence décroissante, vue Kanban desktop 4 colonnes, bouton Voir tout dans les encadrés personnels, et export CSV de la liste filtrée.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Kanban extrait dans lib/widgets/issues/kanban_board.dart. 24 clés ARB ajoutées (FR+EN). flutter analyze passe sans erreur (37 infos pré-existants).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Split View + Actions Superviseur IssueDetail</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Split View Gmail (&gt;=800px) dans IssueTrackingScreen : liste à gauche, IssueDetailScreen en panneau à droite. Bannière RBAC 'Pris en charge par', réassignation et commentaire pour supervisor/admin, timeline HH:mm, section Documents GMAO.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>flutter analyze --no-fatal-infos : 0 erreur. Fix value-&gt;initialValue DropdownButtonFormField. Clés i18n : issueDetailHandledBy, issueDetailReassign*, issueDetailComment*, issueDetailSectionDocuments, issueDetailPanelNoSelection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-016</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Espace Technicien Master-Detail &amp; Timer</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Layout split desktop (&gt;800px), chronomètre live d'intervention (Timer.periodic), sélecteur de pièces depuis inventaire, tooltip sur bouton résolu, agenda fixé sur takenAt</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Refonte ReportsScreen BI</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Ajout filtres temporels (7j/30j/90j/année/custom), KPIs GMAO (MTTR, conformité PM, top 3 depts), export CSV réel, i18n FR+EN</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>StatefulWidget + ListenableBuilder, calcul local sur DataService, export via csv_export.dart, widget ReportKpiSection extrait dans lib/widgets/reports/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-018</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Refonte AnalyticsScreen</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Suppression métriques IT (logins/failed logins), ajout graphiques fl_chart (LineChart tendances 13 semaines, BarChart par groupe technique), correction parsing equipment_by_status (Object→Map), croisement données issues/analytics</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Nouveaux widgets : lib/widgets/analytics/incident_trend_chart.dart, resolution_bar_chart.dart. 16 nouvelles clés i18n (FR+EN). fl_chart ^0.69.0 ajouté au pubspec.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Implement backup restoration functionality with user confirmation and access control
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1098,6 +1098,40 @@
         </is>
       </c>
     </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Sécurisation BackupManagement</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Verrouillage strict rôle admin (RBAC guard dans build), masquage UI déjà assuré par requiredPermission, warning rouge si auto-backup désactivé, double confirmation par frappe RESTAURER avant restauration DB.</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Garde UserRole.admin inviolable. Bouton Restaurer ajouté dans historique. BackupService.restoreBackup() ajouté. 14 nouvelles clés i18n FR+EN.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Refactor login screen to remove signup functionality and add access request feature
- Removed signup mode from authentication flow.
- Added access request dialog for users to request access.
- Updated API service to handle access requests.
- Modified health status indicators for better clarity.
- Enhanced error handling and user feedback in the access request process.
- Updated dependencies in pubspec.yaml and pubspec.lock.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1132,6 +1132,138 @@
         </is>
       </c>
     </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-020</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Audit et MAJ Dépendances</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Mise à jour sécurisée des packages Node.js et Flutter, résolution des alertes d'audit et vérification CI</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>auth-service: express 4.22.2, helmet 8.2.0, jwks-rsa 3.2.2. db-service: axios 1.16.1 (19 CVE résolus), express 4.22.2, helmet 8.2.0. flutter-app: cupertino_icons 1.0.9, shared_preferences 2.5.5. Risques résiduels documentés: tar (build-time/bcrypt) + xlsx (no-fix-available, admin-only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Refonte LoginScreen et Access Request</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Remplacement du signup auto-declaratif par demande d'acces validee par admin, indicateur sante API discret (point colore + tooltip), contact urgence IT, banniere IAM actionnable.</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Nouvel endpoint POST /api/auth/access-request, table access_requests en DB, kDebugMode verifie pour Quick Dev Login.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-022</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Refonte HomeHubScreen par Rôle</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Transformation du hub en dashboard métier : vue actions rapides pour le personnel soignant, plan de travail GMAO pour les techniciens, KPIs + fraîcheur des données pour admins/superviseurs, FAB étendu.</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>RBAC strict : hospitalStaff → gros bouton Signaler + incidents actifs ; technicien* → PM dues/en retard, interventions assignées, pièces en attente ; admin/superviseur → KPIs + indicateur lastRefresh + 3 modules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Refonte DashboardScreen Adaptatif</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>StatCards interactives avec navigation filtrée vers EquipmentListScreen, responsive mobile corrigé (grille 2x2+1), vues par rôles (Météo de l'hôpital pour hospitalStaff, Mes tâches du jour pour techniciens) et auto-refresh Timer.periodic 5 min avec indicateur LinearProgressIndicator.</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Add EquipmentFilterState for managing filter persistence and reset on logout
- Implement EquipmentFilterState as a singleton to manage filter states for EquipmentListScreen.
- Reset filter states upon user logout in AuthService.
- Register new plugins: url_launcher and share_plus for Linux and Windows platforms.
- Update pubspec.yaml and pubspec.lock to include new dependencies.
- Update generated plugin registrants for macOS, Linux, and Windows.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1264,6 +1264,74 @@
       <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="2" t="inlineStr"/>
     </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-024</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Refonte UX EquipmentListScreen</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Filtres persistants via EquipmentFilterState singleton, vue grille/liste desktop, colonnes adaptatives RBAC (Dernière PM pour techniciens), alertes PM inline sans filtre, export CSV mobile via share_plus, scan QR avec MobileScanner, droits édition étendus aux techniciens, filtre unité pour hospitalStaff.</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>7 fonctionnalités GMAO intégrées. share_plus 10.1.4. flutter analyze : 0 erreur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Refonte UX IssueFormScreen</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Formulaire en 2 étapes (catégorie+équipement+urgence / description+photos), urgence sélectionnable dès l'étape 1, mode équipement non répertorié (Bio+IT), guide visuel photos, bouton Scan &amp; Block QR urgence Critique.</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Backend : hasEquipmentName ajouté pour autoriser equipment_name sans equipment_id. Scan &amp; Block saute directement à l'étape 2. i18n : 11 nouvelles clés FR+EN.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Add escalation functionality for technician issues
- Implemented localization strings for English and French related to escalation and work order processes.
- Enhanced the Technician Update Screen to support issue escalation, including UI updates for escalation dialogs and buttons.
- Added backend support for escalating issues via the API, including a new endpoint for handling escalation requests.
- Updated the database service to include methods for escalating issues.
- Improved the handling of work order closures, including the ability to confirm stock deductions for parts used.
- Refactored the available issues display to group by department and show counts of issues per department.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1332,6 +1332,40 @@
         </is>
       </c>
     </row>
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-026</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Refonte TechnicianUpdateScreen (Work Orders)</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Badges d'onglets, chrono persistant (taken_at), déstockage transactionnel avec confirmation, workflow d'escalade (Waiting Materials/Redirected) et tri/groupement par département.</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Backend: migration taken_at, PUT étendu (parts_consumed), PATCH /escalate. Flutter: groupement dept, dialog bon de travail (safety checkbox), dialog destock, dialog escalade.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Add 'Other / Not listed' option for access requests and update dropdowns in access request form
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1366,6 +1366,36 @@
         </is>
       </c>
     </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-027</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Dropdowns département/rôle dans demande d'accès</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Remplacement des champs texte libres département et rôle par des menus déroulants avec la liste des 18 départements de l'hôpital et des 7 rôles système dans le formulaire de demande d'accès.</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Update access request flow to create accounts directly with password and role assignment
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1396,6 +1396,36 @@
       <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr"/>
     </row>
+    <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-028</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Auto-inscription hospitalStaff sans validation admin</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Le formulaire 'Demander un accès' crée maintenant le compte Keycloak immédiatement avec le rôle hospitalStaff. Le dialog se ferme et l'utilisateur est auto-connecté sans intervention admin. Champs mot de passe ajoutés, dropdown rôle supprimé.</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add email notification preferences for users
- Introduced new database tables for role change requests and user notification preferences.
- Implemented API endpoints to get and update user notification preferences.
- Added functionality to send email notifications based on user preferences for various events.
- Created a dialog for users to configure their email notification preferences during first login and in account settings.
- Updated localization files for English and French to support new notification preference texts.
- Enhanced the Flutter app to manage notification preferences and display relevant UI components.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1426,6 +1426,40 @@
       <c r="G29" s="2" t="inlineStr"/>
       <c r="H29" s="2" t="inlineStr"/>
     </row>
+    <row r="30" ht="28" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-029</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Préférences de Notifications Email</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Système permettant aux superviseurs, techniciens et admins de choisir quelles notifications email recevoir. Modal de 1ère connexion, section Settings, endpoints GET/PUT /api/users/me/notifications dans auth-service, table user_notification_preferences, service Brevo et endpoint interne pour db-service.</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Backend: auth-service (DB migration + route notifications + email Brevo + endpoint interne /internal/notifications). Flutter: modèle NotificationPreferences, widget modal, section AccountSettingsScreen, détection 1ère connexion dans main.dart. i18n FR+EN.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Update notification preferences and localization for critical incidents
- Refactored email notification preferences to focus on critical incidents only.
- Updated localization strings for English and French to reflect changes in notification titles and descriptions.
- Added reporter phone number to the Issue model and updated related screens to display contact options.
- Enhanced notification preferences dialog to categorize alerts for technicians and supervisors.
- Integrated URL launcher for direct calling and emailing from the issue detail screen.
- Updated API configuration for feature flags and added feature service for role-based access.
- Added new dependencies for URL launching functionality across platforms.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1460,6 +1460,108 @@
         </is>
       </c>
     </row>
+    <row r="31" ht="28" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-030</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Raccourci appel/email signaleur incident</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Boutons d'appel (tel:) et email (mailto:) dans la page détail d'un incident, sur la ligne du signaleur. reporter_phone ajouté en DB et transmis depuis le formulaire.</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>url_launcher ^6.3.0 ajouté. Fonctionne web (mobile browser) et Android. Sur desktop, le tooltip affiche le numéro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="28" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-031</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Refonte Notifications — Incidents Critiques</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Remplacement des notifications génériques par des alertes ciblées sur les incidents CRITIQUES uniquement : technicien alerté à la création, superviseur alerté à la prise en charge, au diagnostic et à la résolution (avec KPIs : délai, diagnostic, actions, pièces). Suppression des notifications de changement de statut.</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Backend: 4 nouvelles colonnes DB (notify_critical_*), 4 templates HTML Brevo avec KPIs. db-service: 3 déclencheurs dans PUT /api/issues (acknowledged, diagnosed, resolved). Flutter: modèle mis à jour, UI remaniée avec sections Technicien/Superviseur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-032</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Feature Flags et modularite</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Systeme d activation/desactivation des modules (equipment, inventory) par role, avec table feature_flags, endpoints auth-service et navigation dynamique Flutter</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Settings verrouille. Module Inventaire et Equipement desactivables globalement ou par role. 15 tests Jest. flutter analyze OK.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ajout des scénarios de recette pour le contrôle d'accès basé sur les rôles (RBAC) dans le module de gestion des équipements médicaux, incluant des tests pour chaque rôle (hospitalStaff, supervisor, technician, technician_biomedical, technician_it, technician_infra, admin) et des scénarios cross-rôles. Mise à jour du fichier de suivi des vérifications.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1562,6 +1562,142 @@
         </is>
       </c>
     </row>
+    <row r="34" ht="28" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-033</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Scénarios de test RBAC par rôle</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Suite complète de tests manuels (Given-When-Then), Jest backend et flutter_test frontend couvrant les 7 rôles Keycloak et les 14 permissions applicatives</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Scénarios manuels dans tests/scenarios/, Jest dans auth-service/src/tests/ et db-service/src/tests/, widget tests dans flutter-app/test/rbac/ — constat de sécurité documenté : GET /api/inventory sans requireRole backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-034</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Tests widget Flutter RBAC</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Suite de tests flutter_test vérifiant la visibilité conditionnelle des éléments UI selon le rôle : hub screen routing, cartes modules, sidebar, dashboard et permissions AuthService</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Fichier : flutter-app/test/rbac/rbac_visibility_test.dart — 24 tests couvrant 7 groupes. flutter analyze --no-fatal-infos : exit code 0. flutter test bloqué par objective_c native hook (path avec espaces) — passer par CI Jenkins/Docker</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="28" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-035</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Scénarios de test RBAC par rôle — Bilan</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Clôture de la suite RBAC : note de synthèse, plan d'amélioration, 14/14 permissions couvertes, 176 nouveaux tests (73 Jest auth + 79 Jest db + 24 Flutter)</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Lacune documentée : GET /api/inventory sans requireRole backend (ticket ouvert). Tests Flutter bloqués localement (objective_c path spaces), fonctionnels en CI Jenkins/Docker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="28" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-036</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Export PDF ReportsScreen</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Bouton téléchargement PDF sur ReportsScreen avec KPIs GMAO : équipements par statut/département/catégorie, incidents par urgence/statut/catégorie, PM en retard/imminentes, MTTR, inventaire critique. Génération côté client Flutter via PdfReportService (pdf + printing). Option B retenue.</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Accessible aux utilisateurs ayant la permission generateReports (canGenerateReports). Bouton visible conditionnellement. Filtres V1 : période sélectionnée dans l'UI. Correction PdfColors.white70 → PdfColor(0.85,0.85,0.85). flutter analyze --no-fatal-infos : 0 erreur. objective_c native build failure est préexistant (mobile_scanner + local_auth).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Adjust padding and font size in StatusBadge for improved compact display
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1698,6 +1698,36 @@
         </is>
       </c>
     </row>
+    <row r="38" ht="28" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-037</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Ajustement UI statut équipement</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Réduction des marges et du padding du badge de statut dans EquipmentListScreen pour optimiser l'espace d'affichage.</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Enhance equipment maintenance management
- Added new fields to MaintenanceRecord for technicianId, maintenanceType, durationMinutes, and recordId.
- Updated Equipment model to include pmProtocols and pmFrequencyMonths.
- Implemented API endpoints for fetching and updating preventive maintenance plans.
- Created PdfLabelService for generating maintenance labels in PDF format.
- Enhanced EquipmentMaintenanceTab to manage PM frequency, validate maintenance, and print labels.
- Introduced PmChecklistWidget for interactive checklist management during preventive maintenance.
- Updated UI components to reflect changes in maintenance history and compliance rates.
- Modified verification spreadsheet to track changes in maintenance processes.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1860,6 +1860,190 @@
         </is>
       </c>
     </row>
+    <row r="43" ht="28" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-042</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>PM - Checklist interactive</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Widget PmChecklistWidget avec cases à cocher RBAC, compteur de progression et fallback protocole absent. Modèle PmChecklistItem (fromJson multi-format string/map).</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr"/>
+      <c r="G43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>flutter analyze --no-fatal-infos : 0 erreur/warning. Accessible via GlobalKey depuis EquipmentMaintenanceTab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="28" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-043</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>PM - Fréquence de maintenance</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Dropdown fréquence dans onglet GMAO, UPSERT preventive_maintenance_plans via PUT /api/equipment/:id/pm-plan, audit trail. Fréquence persistée depuis pmPlan dans GET /api/equipment/:id.</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="28" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-044</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>PM - Validation officielle</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>POST /maintenance enrichi : snapshot checklist, durée, pièces, calcul next_pm SQLite, déstockage inventaire. Migrations maintenance_records (5 nouvelles colonnes). Flutter : bouton RBAC, dialog confirmation, reload équipement.</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr"/>
+      <c r="G45" s="2" t="inlineStr"/>
+      <c r="H45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46" ht="28" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-045</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>PM - Étiquette PDF</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>PdfLabelService Flutter (pdf+printing, A6 paysage, pattern PdfReportService). GET /api/equipment/:id/maintenance-label/:record_id backend (pdfkit). Bouton Imprimer dans dialog de validation + bouton autonome dans historique PM.</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="2" t="inlineStr"/>
+      <c r="H46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="28" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-046</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>PM - Notification J-7</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Job quotidien pm_reminder_job.js (24h interval, skip en NODE_ENV=test), appel POST /internal/notifications/send-to-roles auth-service type pm_due. Rappels J-7 et J=0 via SQLite date().</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr"/>
+      <c r="G47" s="2" t="inlineStr"/>
+      <c r="H47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48" ht="28" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-047</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>PM - Historique et conformité</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Section historique PM préventives dans onglet GMAO (filtre maintenance_type=preventive, 10 entrées + 'Voir tout'). KPI taux de conformité calculé côté Flutter (fenêtre fréquence+15j de grâce), badge coloré ≥80%/60-79%/&lt;60%.</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr"/>
+      <c r="G48" s="2" t="inlineStr"/>
+      <c r="H48" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add document management features to equipment tab
- Implemented document upload, download, and deletion functionalities for equipment documents.
- Added support for multiple document types: technical, intervention, and certification.
- Introduced a new model for handling equipment documents and issue photos.
- Enhanced issue detail screen to display incident photos with full-screen viewing capability.
- Integrated image compression for uploaded photos to optimize storage.
- Updated localization files for new document-related strings in English and French.
- Added file picker dependency for selecting documents to upload.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2044,6 +2044,156 @@
       <c r="G48" s="2" t="inlineStr"/>
       <c r="H48" s="2" t="inlineStr"/>
     </row>
+    <row r="49" ht="28" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-048</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Docs - Table equipment_documents + endpoints</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Nouvelle table equipment_documents (3 types), multer upload, endpoints GET/POST/download/soft-delete, audit trail</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr"/>
+      <c r="G49" s="2" t="inlineStr"/>
+      <c r="H49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50" ht="28" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-049</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Docs - Table issue_photos + endpoints</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Table issue_photos, upload multipart max 5 photos, endpoint download par incident, audit trail</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr"/>
+      <c r="G50" s="2" t="inlineStr"/>
+      <c r="H50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="28" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-050</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Docs - Onglet Documents Flutter (2 sections + RBAC)</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Widget EquipmentDocumentsTab complet, sections technique/intervention, upload file_picker, RBAC canManageEquipment, ApiClient.postMultipart</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr"/>
+      <c r="G51" s="2" t="inlineStr"/>
+      <c r="H51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52" ht="28" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-051</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Docs - Compression images IssueFormScreen</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>ImageCompressor service (web=bypass natif=placeholder), upload multipart photos après createIssue, max 5 photos</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr"/>
+      <c r="G52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53" ht="28" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-052</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Docs - Photos incidents dans IssueDetailScreen</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Section photos dans fiche incident, modèle IssuePhoto, grille vignettes 1-2 colonnes avec download et préview plein écran</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr"/>
+      <c r="G53" s="2" t="inlineStr"/>
+      <c r="H53" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add issue staff detail screen and enhance issue tracking
- Introduced a new screen for hospital staff to view incident details in read-only mode.
- Updated issue tracking to conditionally navigate to the new detail screen based on user permissions.
- Implemented pagination in the equipment list screen for better data handling.
- Added localization strings for new features in both English and French.
- Enhanced the sidebar to dynamically display subtitles based on the active screen.
- Improved the reports screen with a more responsive layout for mobile devices.
- Updated technician update screen to optimize tab display for mobile users.
- Modified the equipment list screen to include a "Show more" button for pagination.
- Updated the verification Excel file to reflect recent changes.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2194,6 +2194,40 @@
       <c r="G53" s="2" t="inlineStr"/>
       <c r="H53" s="2" t="inlineStr"/>
     </row>
+    <row r="54" ht="28" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-053</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Corrections UX Mobile v3</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Responsivite TechnicianUpdateScreen (TabBar icones sur mobile &lt;600px), ReportsScreen (archives en tete, boutons responsifs), pagination EquipmentList en memoire (pageSize=20, reset sur filtre), titre sidebar dynamique par ScreenType, badge notifications sidebar desktop, vue lecture seule IssueStaffDetailScreen avec timeline horodatee pour hospitalStaff</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr"/>
+      <c r="G54" s="2" t="inlineStr"/>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>6 taches UI Flutter - aucun changement backend ni schema DB - nouvel ecran issue_staff_detail_screen.dart cree (14 ecrans)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add role-based navigation checks for KPI tiles in HomeHubScreen
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2228,6 +2228,40 @@
         </is>
       </c>
     </row>
+    <row r="55" ht="28" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-054</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Fix navigation KPI vers modules désactivés</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Les tuiles KPI du hub (alertes stock, équipements HS) ne naviguent plus vers des modules désactivés dans les settings. onTap mis à null si le module est inaccessible.</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr"/>
+      <c r="G55" s="2" t="inlineStr"/>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Fichier modifié : home_hub_screen.dart — _buildKpiRow et _KpiTile.onTap rendu nullable</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: implement debug notification features including immediate and scheduled notifications
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2262,6 +2262,40 @@
         </is>
       </c>
     </row>
+    <row r="56" ht="28" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-055</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Boutons debug notifications</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Ajout de 2 endpoints backend (notify-now, notify-schedule) et 4 boutons Flutter dans DebugTestScreen pour tester l'envoi de notifications email depuis le panneau admin</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr"/>
+      <c r="G56" s="2" t="inlineStr"/>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Type d'email utilise : critical_new_issue (auth-service). Scheduling in-memory uniquement — reinitialise au redemarrage du serveur. flutter analyze OK.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add push notification banner with activation option and localization support
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2296,6 +2296,36 @@
         </is>
       </c>
     </row>
+    <row r="57" ht="28" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-056</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Bannière push notifications</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Bandeau d'avertissement compact sur HomeHubScreen quand les notifications push ne sont pas activées. Bouton Activer déclenche requestAndSubscribe(), fermeture manuelle possible via X.</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr"/>
+      <c r="G57" s="2" t="inlineStr"/>
+      <c r="H57" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: update stock alert handling based on inventory feature flag
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2326,6 +2326,40 @@
       <c r="G57" s="2" t="inlineStr"/>
       <c r="H57" s="2" t="inlineStr"/>
     </row>
+    <row r="58" ht="28" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-057</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Masquage alertes dashboard selon feature flags</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Les alertes stock (out of stock, low level) du hub principal sont masquées quand le module Inventaire est désactivé dans les feature flags.</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr"/>
+      <c r="G58" s="2" t="inlineStr"/>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>Correction dans home_hub_screen.dart _buildManagerView : stockAlertCount=0 si module inventory désactivé.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Implement responsive design with AppBreakpoints and refactor layout components
- Added AppBreakpoints class for consistent breakpoint management (desktop ≥ 800px, tablet ≥ 600px).
- Refactored user management screen, issue category selector, and report KPI section to use AppBreakpoints.
- Created new layout components: AppSidebar, AppTopBar, and AppBottomNav for better structure and maintainability.
- Introduced TabLabel widget for responsive tab labels, reducing code duplication.
- Cleaned up main.dart and various screens by replacing magic numbers with AppBreakpoints.
- Removed dead code and improved overall code organization for better readability and maintainability.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2360,6 +2360,40 @@
         </is>
       </c>
     </row>
+    <row r="59" ht="28" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-058</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>refactoring-clean-code-global</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Audit et refactoring Clean Code complet : centralisation TECH_ROLES/rolesCsv (5 routes → utils/roles.js), suppression dead code enrichEquipment, AppBreakpoints (18 occurrences), TabLabel widget, NavItem/ScreenType publics, AppSidebar/AppTopBar/AppBottomNav extraits de main.dart, _AvailableIssueCard + helpers top-level depuis TechnicianUpdateScreen</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr"/>
+      <c r="G59" s="2" t="inlineStr"/>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>flutter analyze 0 error 0 warning. npm test 113/113. main.dart réduit de 991 à 436 lignes.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add in-app notifications system with CRUD operations
- Implemented database migration for notifications table with necessary fields and indexes.
- Added API endpoints for fetching, marking notifications as read, and retrieving user-specific notifications.
- Integrated notifications into the debug screen for immediate testing and persistence.
- Enhanced localization files to support new notification strings in English and French.
- Updated notification service to handle fetching from the API and displaying OS notifications.
- Introduced UI components for displaying notifications in the home hub and reports screens with expandable sections.
- Added a new OS notification service for handling platform-specific notifications.
- Updated existing notification model to accommodate new fields from the API.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2394,6 +2394,40 @@
         </is>
       </c>
     </row>
+    <row r="60" ht="28" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-059</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Correctif et OS Notifications</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Ajout cloche HomeHub avec badge, fix flux DebugTestScreen vers notifs in-app, table notifications DB, endpoints GET/PATCH /api/notifications, fetchFromApi dans NotificationService, OsNotificationService stub, i18n 7 clés</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr"/>
+      <c r="G60" s="2" t="inlineStr"/>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Table notifications créée dans hospital.db via migration idempotente. Cloche visible dans HomeHubScreen._buildHeader. DebugTestScreen appelle fetchFromApi après notify-now. Endpoints ajoutés dans push_notifications.js sur /api/notifications existant.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add Departments and Roles management tabs
- Implement DepartmentsTab for managing departments with search, add, edit, and delete functionalities.
- Create RolesTab for managing user roles, including permissions and sidebar order configuration.
- Add localization support for new UI elements and actions.
- Update verification spreadsheet to reflect recent changes.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2428,6 +2428,36 @@
         </is>
       </c>
     </row>
+    <row r="61" ht="28" customHeight="1">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-060</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Refonte UI Administration</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Refonte du SettingsScreen : 4 onglets NavigationRail (Départements CRUD API-backed + stats, Catégories arborescence macro/sub, Rôles &amp; Permissions + Ordre menu fusionnés, Journal d'activité paginé). Backend : routes CRUD /api/departments + POST/PUT/DELETE /api/categories/sub. Seed 18 départements hôpital.</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr"/>
+      <c r="G61" s="2" t="inlineStr"/>
+      <c r="H61" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Add role detail screen with hierarchy, permissions, sidebar order, and user management
- Implemented GET endpoints for role permissions and hierarchy in auth-service.
- Added role detail screen in Flutter app with tabs for hierarchy, features, menu, and users.
- Introduced RoleDetailConfig and RoleUserSummary models for managing role data.
- Enhanced localization for role detail features in English and French.
- Integrated role detail navigation from roles tab with a "Details" button.
- Added API service methods for fetching role hierarchy, permissions, and users.
- Implemented sidebar order management for roles.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2458,6 +2458,36 @@
       <c r="G61" s="2" t="inlineStr"/>
       <c r="H61" s="2" t="inlineStr"/>
     </row>
+    <row r="62" ht="28" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-061</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Role Detail Screen &amp; Hiérarchie</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Page de configuration dédiée par rôle (4 onglets : hiérarchie parent/enfant, permissions, ordre menu sidebar, utilisateurs). Table role_hierarchy SQLite + 3 endpoints GET backend. Navigation depuis l'onglet Rôles des Paramètres.</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr"/>
+      <c r="G62" s="2" t="inlineStr"/>
+      <c r="H62" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Implement biomedical replacement plan feature (RA3 S5)
- Added functionality to export a PDF report for the biomedical replacement plan.
- Created a new screen for subcategory details, displaying alerts for equipment needing replacement.
- Introduced a new badge widget to indicate replacement status with tooltips.
- Updated API service to handle fetching and updating expected lifespan for subcategories.
- Enhanced the PDF report service to include detailed tables and KPIs for the replacement plan.
- Modified the app theme to include colors for replacement status badges.
- Implemented RBAC for accessing replacement plan features and lifespan updates.
- Added localization support for new UI strings related to the replacement plan.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2556,6 +2556,40 @@
         </is>
       </c>
     </row>
+    <row r="65" ht="28" customHeight="1">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-064</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Plan de remplacement biomédical</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Durée de vie de référence par sous-catégorie + calcul serveur statut/horizon + écran gestion sous-catégories + page détail + badges triangle + section notifications + rapport PDF plan de remplacement (RA3 S5)</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr"/>
+      <c r="G65" s="2" t="inlineStr"/>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>Endpoints GET /api/equipment/replacement-plan (admin/supervisor), PUT /api/categories/sub/:id/lifespan (admin). 19 tests calcul. flutter analyze sans erreur.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add intervention report section and related functionalities
- Introduced InterventionReportSection widget for managing intervention reports.
- Implemented loading, editing, saving, finalizing, and reopening of reports.
- Added PDF generation and archiving capabilities for finalized reports.
- Enhanced issue detail screens to include intervention report section for hospital staff and admin users.
- Updated reports screen to compute and display maintenance costs alongside MTTR.
- Added new API endpoints for fetching, saving, finalizing, and reopening intervention reports.
- Updated PDF report generation to include maintenance cost information.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2684,6 +2684,36 @@
         </is>
       </c>
     </row>
+    <row r="69" ht="28" customHeight="1">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-068</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Rapport d'intervention par incident</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Rapport structure editable 1:1 par incident (resume, cause racine, recommandations, duree, cout, etat final, signatures), fige a la cloture, export PDF + archivage auto dans l'historique equipement, branche MTTR/cout</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr"/>
+      <c r="G69" s="2" t="inlineStr"/>
+      <c r="H69" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Implement clickable metadata in equipment detail screen with breadcrumb navigation
- Added detailSectionHeader and detailEmptyCard helper functions to detail_screen_helpers.dart for reusable UI components.
- Enhanced EquipmentDetailScreen to include breadcrumb navigation for department, subcategory, and equipment.
- Updated EquipmentInfoTab to support clickable links for department, category, subcategory, manufacturer, and model based on availability.
- Created DetailBreadcrumb widget for consistent breadcrumb display across detail screens.
- Introduced new API endpoints for fetching department and category details.
- Updated DbApiService to handle new API calls for department and category details.
- Modified existing models and services to accommodate new fields for equipment metadata.
- Ensured internationalization support for new UI elements and API responses.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2714,6 +2714,40 @@
       <c r="G69" s="2" t="inlineStr"/>
       <c r="H69" s="2" t="inlineStr"/>
     </row>
+    <row r="70" ht="28" customHeight="1">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-069</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Métadonnées cliquables fiche équipement</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Drill-down depuis la fiche équipement vers sous-catégorie/fabricant/modèle/catégorie/département + breadcrumb cliquable sur toutes les fiches de détail (vue complète)</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr"/>
+      <c r="G70" s="2" t="inlineStr"/>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>Backend lecture seule (BASE_SELECT enrichi brand_id/brand_name, GET /api/categories/detail, GET /api/departments/:id/detail). 2 nouveaux écrans Flutter. 6 tests Jest.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Enhance department dashboard with resolved issues and localization updates
- Updated database schema to include location_text, location_tag, and taken_at fields in issues.
- Modified department detail route to fetch and return resolved issues alongside open issues.
- Updated frontend to display ongoing and resolved issues in the department detail screen.
- Improved localization for English and French languages, including new keys for resolved issues and incident categories.
- Enhanced issue list display to show location names and categories for better clarity.
- Updated tests to cover new functionality for resolved issues and localization changes.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2748,6 +2748,70 @@
         </is>
       </c>
     </row>
+    <row r="71" ht="28" customHeight="1">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-070</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Déploiement IP-only par défaut</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Bascule du chemin de déploiement par défaut sur IP publique brute + certificat auto-signé ; retrait des références codées en dur à kabutare.duckdns.org (config.js, CLAUDE.md, contexte.md, plan.md, fixtures). Famille domaine conservée mais débranchée.</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr"/>
+      <c r="G71" s="2" t="inlineStr"/>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>config.js BREVO_SENDER_EMAIL -&gt; noreply@hospital.local ; plan.md réécrit autour de setup_ubuntu.sh ; limitation SPF/DKIM documentée. npm test auth-service: 166/166 OK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="28" customHeight="1">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-071</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Incidents par département + téléchargement rapport finalisé</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Page détail département : KPI incidents ouverts, sections en cours/résolus avec badge catégorie + cible (équipement/lieu) cliquables ; dialogue de téléchargement du PDF à la finalisation du rapport d'intervention</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr"/>
+      <c r="G72" s="2" t="inlineStr"/>
+      <c r="H72" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add clickable urgent alerts and quick action for technicians
- Implemented clickable `EquipmentCriticalBanner` to navigate to the Incidents tab.
- Added `takeOverIssue` method in `DbApiService` to allow technicians to take over incidents.
- Updated `AlertCard` to include navigation for urgent alerts on the dashboard.
- Refactored `dashboard_screen.dart` to wire up the new functionality for urgent alerts.
- Created detailed prompts for urgent alerts and technician page redesign.
- Added a new `TechnicianScheduleScreen` for better scheduling management.
- Enhanced validation process in `technician_update_screen.dart` for incident handling.
- Updated localization files for new strings related to the changes.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2812,6 +2812,66 @@
       <c r="G72" s="2" t="inlineStr"/>
       <c r="H72" s="2" t="inlineStr"/>
     </row>
+    <row r="73" ht="28" customHeight="1">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-072</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Alertes urgentes cliquables + prise en charge rapide</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Drill-down des AlertCard dashboard + banniere critique vers onglet Incidents + bouton Prendre en charge technicien sur incidents prioritaires</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr"/>
+      <c r="G73" s="2" t="inlineStr"/>
+      <c r="H73" s="2" t="inlineStr"/>
+    </row>
+    <row r="74" ht="28" customHeight="1">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-073</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Refonte page technicien</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Onglet A valider en premier, planning en page separee, validation+reassignation deleguees au detail d'incident (bouton Examiner), delai de signalement affiche</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr"/>
+      <c r="G74" s="2" t="inlineStr"/>
+      <c r="H74" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Delete obsolete prompt files for incident intervention report, technician page redesign, and modifications by page. Update verification tracking spreadsheet to reflect recent changes.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2872,6 +2872,70 @@
       <c r="G74" s="2" t="inlineStr"/>
       <c r="H74" s="2" t="inlineStr"/>
     </row>
+    <row r="75" ht="28" customHeight="1">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-074</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Suivi incidents 3 onglets</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Refonte IssueTrackingScreen en 3 onglets (Mes signalements / Tous actifs / Terminés), suppression split view, clic ouvre la page détail, colonne resolved_at backend</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr"/>
+      <c r="G75" s="2" t="inlineStr"/>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>Flutter + db-service. Tabs avec badges compteurs, date de résolution sur onglet Terminés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="28" customHeight="1">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-075</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Ré-agencement cartes page Rapports</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Appairage Breakdown by status + Issue statistics, et Equipment by department + Equipment by category, dans les deux LayoutBuilder de ReportsScreen (responsive conservé).</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr"/>
+      <c r="G76" s="2" t="inlineStr"/>
+      <c r="H76" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Enhance Equipment Info and Maintenance Tabs
- Updated EquipmentInfoTab to include critical banner, state summary, and consolidated notifications.
- Added field editing capabilities for various equipment attributes based on user roles.
- Improved notification handling for maintenance alerts and replacement statuses.
- Refactored inventory card and tags display for better clarity and usability.
- Removed standalone PM alert banner from EquipmentMaintenanceTab; integrated alerts into EquipmentInfoTab.
- Enhanced maintenance record dialog to include detailed information and label printing options.
- Updated PM history row to allow for detailed maintenance record viewing.
- Modified Excel verification file for tracking changes.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2936,6 +2936,40 @@
       <c r="G76" s="2" t="inlineStr"/>
       <c r="H76" s="2" t="inlineStr"/>
     </row>
+    <row r="77" ht="28" customHeight="1">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-076</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Refonte fiche équipement (4 onglets)</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Onglet Info: édition par champ inline, description sous-cat, résumé d'état, notifications cliquables (durée de vie/incident/PM/remplacement), QR+étiquette PM. Maintenance: section PM réagencée, historique cliquable + étiquette d'époque. Notifications retirées des autres onglets.</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr"/>
+      <c r="G77" s="2" t="inlineStr"/>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>Nouvelle colonne equipment_subcategories.description (migration idempotente).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor equipment list screen to remove edit button; enhance issue form with building and location fields; update issue tracking screen to use nested scroll view; add role request dialog for role selection after account creation; implement subcategory management with edit and delete functionality; improve status badge with tooltip and text overflow handling; add database reseed functionality for admin; update authentication service to manage role selection state; modify categories tab to streamline UI and remove unused code.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2970,6 +2970,224 @@
         </is>
       </c>
     </row>
+    <row r="78" ht="28" customHeight="1">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-077</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Audit volume flux de connexion</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Audit lecture seule du volume de donnees (bundle web + payloads API du login) du premier acces sur dev.app.lucaslopvet.fr, profils admin et hospitalStaff, recommandations bas-debit chiffrees</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr"/>
+      <c r="G78" s="2" t="inlineStr"/>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>Lecture seule, aucune modif de code</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="28" customHeight="1">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-078</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Correction badge statut + retrait modif inline liste equipements</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Fix overflow visuel StatusBadge (ellipsis + tooltip) et suppression des 3 boutons Modifier redondants dans l'onglet Liste equipements (modification conservee uniquement sur la fiche detail)</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr"/>
+      <c r="G79" s="2" t="inlineStr"/>
+      <c r="H79" s="2" t="inlineStr"/>
+    </row>
+    <row r="80" ht="28" customHeight="1">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-079</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Alerte sous-catégorie vide + actions déplacées vers fiche détail</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Icône d'alerte si equipment_count=0 dans la liste des sous-catégories ; Modifier/Supprimer une sous-catégorie déplacés de l'onglet Catégories vers subcategory_detail_screen.dart (pattern brand_detail_screen)</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr"/>
+      <c r="G80" s="2" t="inlineStr"/>
+      <c r="H80" s="2" t="inlineStr"/>
+    </row>
+    <row r="81" ht="28" customHeight="1">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-080</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Localisation incident + filtres scrollables</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Champs Bâtiment/Lieu précis ajoutés aux onglets Bio/IT/Autre du formulaire d'incident ; bloc filtres de la page de suivi rendu scrollable avec la liste (NestedScrollView)</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr"/>
+      <c r="G81" s="2" t="inlineStr"/>
+      <c r="H81" s="2" t="inlineStr"/>
+    </row>
+    <row r="82" ht="28" customHeight="1">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-081</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Popup sélection de rôle post-création de compte</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Renommage 'Demander un accès' -&gt; 'Créer un compte' ; popup obligatoire de sélection de rôle (technicien/superviseur/garder hospitalStaff) affiché une fois après création de compte, réutilisable depuis Paramètres</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr"/>
+      <c r="G82" s="2" t="inlineStr"/>
+      <c r="H82" s="2" t="inlineStr"/>
+    </row>
+    <row r="83" ht="28" customHeight="1">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-082</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Suppression blocage email non vérifié</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>Retrait de requiredActions VERIFY_EMAIL à la création de compte (register + access-request) ; script one-shot de déblocage des comptes existants</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr"/>
+      <c r="G83" s="2" t="inlineStr"/>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>Bannières informatives conservées, emailVerified reste false, aucun changement Flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="28" customHeight="1">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-083</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Reset BDD démo (page Debug) + fix bug --dry-run imports</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Bouton admin Réinitialiser la base de données (équipements/incidents/inventaire/lieux) dans le module Debug, appelant POST /api/debug/reseed (seed.js refactorisé en fonction exportable). Corrige aussi le bug de config.js qui rendait --dry-run inopérant sur import_inventory.js et import_infra_inventory.js (lecture tardive de process.env.DB_PATH).</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr"/>
+      <c r="G84" s="2" t="inlineStr"/>
+      <c r="H84" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(settings): add AppSettingsTab for managing general settings including Brevo configuration
feat(status-badge): add support for 'Rejected' status in IssueStatusBadge with appropriate color coding

chore: update verification spreadsheet with new data
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H84"/>
+  <dimension ref="A1:H87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3188,6 +3188,100 @@
       <c r="G84" s="2" t="inlineStr"/>
       <c r="H84" s="2" t="inlineStr"/>
     </row>
+    <row r="85" ht="28" customHeight="1">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-084</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Validation rapide incident + statut Rejected + détachement</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Sheet responsive de validation (signaleur, objet, photos, antécédents) avec valider/rejeter(motif)/réassigner groupe ; statut Rejected ; PATCH /reject &amp; /detach ; détachement technicien retour au pool</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr"/>
+      <c r="G85" s="2" t="inlineStr"/>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>Testé Chrome + Android. Réassignation = groupe uniquement. Pas de migration DB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="28" customHeight="1">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-085</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Page Paramètres application (Settings)</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Onglets Feature Flags + Paramètres généraux ; table app_settings (contact login public + config Brevo base/env, clé masquée) ; email de test ; suppression de l'écran feature flags autonome</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr"/>
+      <c r="G86" s="2" t="inlineStr"/>
+      <c r="H86" s="2" t="inlineStr"/>
+    </row>
+    <row r="87" ht="28" customHeight="1">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-086</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Régénération BDD depuis fichier XLSX (page Debug)</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Bouton admin upload .xlsx (format Equipment Migration Template) qui vide équipements/incidents puis réimporte intégralement via POST /api/debug/reseed-from-file, en réutilisant seedReferences/importEquipment de import_inventory.js. Complète le bouton de reset démo existant.</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr"/>
+      <c r="G87" s="2" t="inlineStr"/>
+      <c r="H87" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(auth): add phone number field to access request and update related logic
- Added phone number field to the access request API and database schema.
- Updated validation for phone number format in the access request form.
- Enhanced localization for phone number prompts in English and French.
- Modified issue tracking and home hub screens to filter issues by department.
- Improved UI components to handle new phone number data.
- Added tests to verify phone number handling in access requests.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H87"/>
+  <dimension ref="A1:H89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3282,6 +3282,66 @@
       <c r="G87" s="2" t="inlineStr"/>
       <c r="H87" s="2" t="inlineStr"/>
     </row>
+    <row r="88" ht="28" customHeight="1">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-087</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Téléphone optionnel à la création de compte</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Champ téléphone optionnel ajouté au formulaire Demande d'accès, propagé à Keycloak et tracé dans access_requests.phone</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr"/>
+      <c r="G88" s="2" t="inlineStr"/>
+      <c r="H88" s="2" t="inlineStr"/>
+    </row>
+    <row r="89" ht="28" customHeight="1">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-088</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Correctifs parcours hospitalStaff</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Fix departement vide signalement non repertorie, navigation My active incidents -&gt; Issue Tracking, filtre+compteur incidents par departement, masquage rapport intervention/export CSV pour hospitalStaff</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr"/>
+      <c r="G89" s="2" t="inlineStr"/>
+      <c r="H89" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(technician): add navigation to issue detail screen from available issue card
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H89"/>
+  <dimension ref="A1:H90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3342,6 +3342,36 @@
       <c r="G89" s="2" t="inlineStr"/>
       <c r="H89" s="2" t="inlineStr"/>
     </row>
+    <row r="90" ht="28" customHeight="1">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-089</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Carte incident disponible cliquable</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Clic sur la carte de l'onglet Disponibles (page technicien) ouvre IssueDetailScreen en consultation, sans impacter les boutons Prendre en charge / Feuille de details</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr"/>
+      <c r="G90" s="2" t="inlineStr"/>
+      <c r="H90" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Add equipment linking functionality and improve photo upload handling
- Added localization strings for linking equipment in English and French.
- Implemented `linkEquipment` method in `DbApiService` to associate equipment with issues.
- Introduced `EquipmentPickerField` widget for selecting equipment in forms.
- Enhanced `IssueFormScreen` to handle photo uploads with retry logic and display error messages.
- Integrated auto-refresh functionality in `DashboardScreen` and `IssueTrackingScreen`.
- Created `AutoRefreshMixin` for periodic refresh capabilities in stateful widgets.
- Updated image compression logic to handle uploads more efficiently.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H90"/>
+  <dimension ref="A1:H92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3372,6 +3372,70 @@
       <c r="G90" s="2" t="inlineStr"/>
       <c r="H90" s="2" t="inlineStr"/>
     </row>
+    <row r="91" ht="28" customHeight="1">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-090</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Fix refresh technicien + photos incident perdues</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Polling 5min sur IssueTrackingScreen + gestion erreur Multer + visibilite echec upload photo + vraie compression image (cause racine)</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr"/>
+      <c r="G91" s="2" t="inlineStr"/>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>Cause racine confirmee par lecture de code : ImageCompressor.compress() etait un placeholder no-op (web ET natif), renvoyant les bytes originaux sans jamais compresser. Une photo de smartphone (souvent 3-12 Mo) depassait donc systematiquement la limite serveur MAX_PHOTO_MB=5 (db-service/src/middleware/upload.js), Multer rejetait le fichier, et l'erreur etait avalee silencieusement cote Flutter (catch vide) + cote serveur renvoyait une page HTML 500 brute (pas de middleware d'erreur Express). Corrige : implementation reelle de la compression via package:image (deja present en transitif, pur Dart, fonctionne web+natif), ajout du middleware d'erreur Multer global, et affichage explicite + bouton Reessayer dans le dialogue de succes si l'upload photo echoue malgre tout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="28" customHeight="1">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-091</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Liaison tardive équipement-incident</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>PATCH /api/issues/:id/link-equipment + UI technicien pour rattacher un équipement à un incident créé sans équipement, avec horodatage equipment_linked_at</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr"/>
+      <c r="G92" s="2" t="inlineStr"/>
+      <c r="H92" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update suivi_verifications.xlsx with new verification data
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H92"/>
+  <dimension ref="A1:H93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3436,6 +3436,36 @@
       <c r="G92" s="2" t="inlineStr"/>
       <c r="H92" s="2" t="inlineStr"/>
     </row>
+    <row r="93" ht="28" customHeight="1">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-092</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Page dédiée mise à jour intervention technicien</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Liste cliquable ouvrant une page séparée (plus de master-detail latéral) ; masquage réactif du sélecteur de pièces si module Inventaire désactivé ; garde-fou anti-perte de saisie</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr"/>
+      <c r="G93" s="2" t="inlineStr"/>
+      <c r="H93" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Add error message for manual report creation when auto-generation fails
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H93"/>
+  <dimension ref="A1:H94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3466,6 +3466,36 @@
       <c r="G93" s="2" t="inlineStr"/>
       <c r="H93" s="2" t="inlineStr"/>
     </row>
+    <row r="94" ht="28" customHeight="1">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-093</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Rapport intervention auto à la clôture</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Génération et finalisation automatique du rapport d'intervention (table issue_intervention_reports) à la clôture du Bon de Travail technicien, mapping depuis diagnostic/actions/chronomètre, PDF archivé sur l'équipement si applicable</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr"/>
+      <c r="G94" s="2" t="inlineStr"/>
+      <c r="H94" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add role request management to user management screen
- Introduced a new model `_RoleRequest` to handle role requests.
- Implemented loading and displaying of role requests in the user management screen.
- Added functionality to approve or reject role requests with a confirmation dialog.
- Enhanced data service to fetch role requests from the API.
- Updated notification service to include role request notifications.
- Created a new widget `InterventionSessionsTimeline` to display intervention sessions.
- Added PDF report generation for intervention sessions.
- Updated notification bell to handle role request notifications.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H94"/>
+  <dimension ref="A1:H97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3496,6 +3496,104 @@
       <c r="G94" s="2" t="inlineStr"/>
       <c r="H94" s="2" t="inlineStr"/>
     </row>
+    <row r="95" ht="28" customHeight="1">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-094</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>Visibilité admin demandes de rôle</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>Notification cloche + section dédiée dans l'écran Users pour les role_change_requests en attente, mirroir du pattern department_change_requests, avec badge d'ancienneté</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr"/>
+      <c r="G95" s="2" t="inlineStr"/>
+      <c r="H95" s="2" t="inlineStr"/>
+    </row>
+    <row r="96" ht="28" customHeight="1">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-095</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Boucles d'intervention multi-passages</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Table issue_intervention_sessions 1:N, rapport PDF par boucle, suivi cliquable sur fiche incident technicien</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr"/>
+      <c r="G96" s="2" t="inlineStr"/>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>3 routes backend + 13 tests Jest, modele Flutter IssueInterventionSession, widget InterventionSessionsTimeline, PDF PdfReportService.generateInterventionSessionReport</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="28" customHeight="1">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-096</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>Simplification — boucles intervention</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Refactor qualité : helper _s() PDF promu statique, appendLine dans issues.js, hasRole() dans utils/roles.js, _buttonSpinner() Flutter, note TODO sur _notifyUser.</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr"/>
+      <c r="G97" s="2" t="inlineStr"/>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>5 fixes simplification/réutilisation. flutter analyze --no-fatal-infos passe (105 info pré-existants, 0 error/warning).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add building and tag number fields to equipment management
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H97"/>
+  <dimension ref="A1:H98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3594,6 +3594,36 @@
         </is>
       </c>
     </row>
+    <row r="98" ht="28" customHeight="1">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-097</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Formulaire équipement enrichi</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Dropdowns brand/model en cascade avec création inline, tag physique (equipment_tags), champ building, toggle PM avec pré-remplissage fréquence depuis le protocole du modèle sélectionné</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr"/>
+      <c r="G98" s="2" t="inlineStr"/>
+      <c r="H98" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update verification spreadsheet with new data and adjustments
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H98"/>
+  <dimension ref="A1:H99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3624,6 +3624,40 @@
       <c r="G98" s="2" t="inlineStr"/>
       <c r="H98" s="2" t="inlineStr"/>
     </row>
+    <row r="99" ht="28" customHeight="1">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-098</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>Seed db-service avec inventaire réel 2025-2026</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>Remplacement de seed.js (db-service) par des données réelles : 338 équipements (tags réels) issus de l'inventaire physique XLSX, 173 enregistrements de maintenance issus du plan PPM Q1+Q2, issues ré-ancrées sur de vrais équipements</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr"/>
+      <c r="G99" s="2" t="inlineStr"/>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>Fichier combiné inventaire (Maternity/Neonatology/Pharmacy etc.) écarté : structure corrompue/incohérente (colonnes décalées en fin de fichier), non hardcodé. locations[] et inventory[] consommables conservés inchangés, aucun des 3 fichiers source ne couvrant ces 2 tables. npm test : 223/223 OK.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add approveRequests permission to technician roles and update related tests
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H99"/>
+  <dimension ref="A1:H100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3658,6 +3658,36 @@
         </is>
       </c>
     </row>
+    <row r="100" ht="28" customHeight="1">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-099</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Validation incidents par techniciens</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Permission approveRequests étendue aux 4 rôles technicien (Reported→Acknowledged), sans filtre groupe ni criticité</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr"/>
+      <c r="G100" s="2" t="inlineStr"/>
+      <c r="H100" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: update technician intervention screen with new save button functionality and localization updates
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H100"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3688,6 +3688,36 @@
       <c r="G100" s="2" t="inlineStr"/>
       <c r="H100" s="2" t="inlineStr"/>
     </row>
+    <row r="101" ht="28" customHeight="1">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-100</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>Fusion Save / Save-and-Close</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>Un seul bouton ElevatedButton ferme toujours la session active ; toggle conditionnel _planNextAction pour next_actions optionnel sans validation minimum</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="E101" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr"/>
+      <c r="G101" s="2" t="inlineStr"/>
+      <c r="H101" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Enhance Issue Form and Technician Update Screens
- Added 'Other' option to infrastructure category selection in Issue Form.
- Adjusted logic to conditionally display subcategory and specific issue fields based on 'Other' selection.
- Updated validation to accommodate the new 'Other' category in the Issue Form.
- Modified technician update logic to filter incidents based on technician's assigned groups.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H101"/>
+  <dimension ref="A1:H104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3718,6 +3718,104 @@
       <c r="G101" s="2" t="inlineStr"/>
       <c r="H101" s="2" t="inlineStr"/>
     </row>
+    <row r="102" ht="28" customHeight="1">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-101</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Option Autre catégorie Infrastructure</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Ajout option Autre dans le dropdown catégorie du Tab Infrastructure pour permettre de signaler un incident hors catalogue, masquage des dropdowns sous-catégorie et problème spécifique</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr"/>
+      <c r="G102" s="2" t="inlineStr"/>
+      <c r="H102" s="2" t="inlineStr"/>
+    </row>
+    <row r="103" ht="28" customHeight="1">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-102</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>Fix onglet À valider techniciens</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>_openIssuesForValidation incluait uniquement admin/supervisor ; ajout du filtre par groupe (Biomédical/IT/Infrastructure) pour les techniciens disposant de la permission approveRequests</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="E103" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr"/>
+      <c r="G103" s="2" t="inlineStr"/>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>technician_update_screen.dart:124-141</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="28" customHeight="1">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-103</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Intégration inventaire combiné (lits/mobilier) dans seed.js</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>Ajout des 542 actifs supplémentaires (hors doublons) issus de 'INVENTORY combined october.xlsx' au seed db-service, avec parsing robuste par classification de cellule (colonnes décalées à partir de la section Pharmacie). Total equipment[] : 880 (338 biomédical + 542 mobilier/divers). Maintenance records enrichis à 188 grâce aux nouveaux noms d'équipement disponibles pour le matching PPM.</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="E104" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr"/>
+      <c r="G104" s="2" t="inlineStr"/>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>Correctif d'un bug de parsing initial (colonne NO confondue avec QTY, faussant serial_number) détecté et corrigé avant intégration finale. npm test : 223/223 OK.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Add intervention document management and localization
- Introduced new localization strings for common actions and intervention document management in both English and French.
- Implemented a new `InterventionDocumentsSection` widget to display and manage intervention-related documents.
- Enhanced the `Issue` model to include a count of archived intervention documents.
- Updated the API client and database service to support uploading and retrieving intervention documents.
- Added functionality for technicians to attach additional documents (PDF/JPEG/PNG) to incidents.
- Implemented a documented closure rate calculation for reports, reflecting the percentage of closed incidents with archived documents.
- Updated various screens and reports to incorporate the new document management features and display relevant information.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H104"/>
+  <dimension ref="A1:H106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3816,6 +3816,70 @@
         </is>
       </c>
     </row>
+    <row r="105" ht="28" customHeight="1">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-104</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Fix fermeture session intervention</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>Save and close créait/mettait à jour la session active via PUT sessions/active avant le POST sessions/active/close, évitant l'erreur 400 'Aucune session active' quand la dialog Compléter le diagnostic n'avait jamais été ouverte</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="E105" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr"/>
+      <c r="G105" s="2" t="inlineStr"/>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>technician_intervention_update_screen.dart _doSaveAndClose</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="28" customHeight="1">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-105</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Documents PDF d'intervention</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>Visualisation PDF a la cloture, upload complementaire multi-fichiers, remplacement du rapport d'intervention manuel par la liste des documents reels, badge + KPI taux de cloture documentee</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="E106" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr"/>
+      <c r="G106" s="2" t="inlineStr"/>
+      <c r="H106" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(api): implement conditional ETag caching for GET requests
- Added support for conditional GET requests in ApiClient with ETag caching.
- Introduced methods to read, write, and clear ETag cache.
- Updated getEquipment and getLocations methods in DbApiService to utilize ETag caching.
- Added pagination support for equipment and issues with PagedResult class.
- Created a new PaginationFooter widget for server pagination UI.
- Updated Nginx configuration for better asset caching and compression settings.
- Added a new sidebar API endpoint to fetch all sidebar configurations in one request.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H106"/>
+  <dimension ref="A1:H108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3880,6 +3880,66 @@
       <c r="G106" s="2" t="inlineStr"/>
       <c r="H106" s="2" t="inlineStr"/>
     </row>
+    <row r="107" ht="28" customHeight="1">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-106</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Bouton Actualiser + pagination serveur</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>Pagination serveur (page/limit/search) sur GET /api/equipment et GET /api/issues, bouton Actualiser sur Équipements/Suivi incidents/Interventions technicien, cache DataService global inchangé</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="E107" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr"/>
+      <c r="G107" s="2" t="inlineStr"/>
+      <c r="H107" s="2" t="inlineStr"/>
+    </row>
+    <row r="108" ht="28" customHeight="1">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-107</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Réduction flux premier accès</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>Compression nginx JS/WASM + cache immutable assets, middleware compression API, payload light equipment, fusion 6 requêtes sidebar, cache conditionnel If-None-Match/304 — premier accès ~11 Mo → ~3,6 Mo (estimé, code prêt mais non déployé)</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr"/>
+      <c r="G108" s="2" t="inlineStr"/>
+      <c r="H108" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(debug): implement debug mode unlock functionality with rate limiting and localization
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H108"/>
+  <dimension ref="A1:H109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3940,6 +3940,36 @@
       <c r="G108" s="2" t="inlineStr"/>
       <c r="H108" s="2" t="inlineStr"/>
     </row>
+    <row r="109" ht="28" customHeight="1">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-108</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>Verrouillage mode Debug &amp; Test</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>Mot de passe admin defini au deploiement (setup_ubuntu.sh, partage prod/dev via /etc/kabutare/.env), requis en plus de Permission.manageFeatures pour afficher l'item sidebar Debug &amp; Test</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr"/>
+      <c r="G109" s="2" t="inlineStr"/>
+      <c r="H109" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor role management and settings screens
- Removed the activity log tab from settings and its associated widget.
- Consolidated role permissions and sidebar order management into a single structure.
- Updated localization files to reflect changes in role detail and settings screens.
- Added a new "Page Access" tab in the role detail screen to manage permissions by module.
- Adjusted the settings screen to remove the activity log and streamline the tab structure.
- Enhanced the UI for better organization and clarity in role and permission management.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H109"/>
+  <dimension ref="A1:H110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3970,6 +3970,40 @@
       <c r="G109" s="2" t="inlineStr"/>
       <c r="H109" s="2" t="inlineStr"/>
     </row>
+    <row r="110" ht="28" customHeight="1">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-109</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Réorganisation Roles &amp; Permissions + page Admin</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>Déplacement Page Access by Role dans le détail de rôle (trié par module), suppression Menu Order dupliqué et onglet Activity Log redondant, en-tête page Admin repliable au scroll</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr"/>
+      <c r="G110" s="2" t="inlineStr"/>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>Aucun changement backend ; corrige au passage la non-persistance des checkboxes de permission de l'ancienne section Page Access</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(pdf): update PDF report generation to include hospital logo and improve localization
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H110"/>
+  <dimension ref="A1:H112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4004,6 +4004,70 @@
         </is>
       </c>
     </row>
+    <row r="111" ht="28" customHeight="1">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-110</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>Filtrage timeline incident photos</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Exclusion des actions techniques upload_issue_photos/download_issue_photo de la timeline d'audit d'un incident (GET /api/issues/:id), sans impact sur l'audit trail global</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="E111" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr"/>
+      <c r="G111" s="2" t="inlineStr"/>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>Modification SQL uniquement, db-service/src/routes/issues.js lignes 212-218</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="28" customHeight="1">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-111</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>Rapports PDF GMAO en anglais + letterhead + numéro de référence</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>Traduction complète des 4 générateurs PDF (pdf_report_service.dart) en anglais fixe, ajout logo + adresse officielle (Southern Province / Huye District / Kabutare District Hospital / P.O. Box 621 Butare / Email), ajout numéro de référence unique par rapport</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr"/>
+      <c r="G112" s="2" t="inlineStr"/>
+      <c r="H112" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Add support for closing equipment as disposed with reason and method selection
- Introduced new localization strings for the "Close as Disposed" feature in both English and French.
- Updated the EquipmentDocument model to include issue-related fields (issueId, issueStatus, issueCreatedAt).
- Modified NotificationPreferences to support new issue notifications with customizable urgency thresholds.
- Implemented UI changes in the Technician Intervention Update screen to include a button for closing equipment as disposed.
- Added a dialog for confirming the closure of equipment as disposed, including fields for reason and disposal method.
- Updated the API service to handle the closure of issues as disposed.
- Enhanced PDF report generation to include issue references.
- Refactored document handling in the Equipment Documents tab to group intervention documents by issue.
- Updated notification preferences dialog to include urgency threshold selection for new issue notifications.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H112"/>
+  <dimension ref="A1:H116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4068,6 +4068,126 @@
       <c r="G112" s="2" t="inlineStr"/>
       <c r="H112" s="2" t="inlineStr"/>
     </row>
+    <row r="113" ht="28" customHeight="1">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-112</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>Seuil urgence notification technicien</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>Sélecteur de niveau d'urgence minimal (Faible/Moyen/Urgent/Critique) à côté du switch email 'nouvel incident' dans les préférences de notification technicien</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr"/>
+      <c r="G113" s="2" t="inlineStr"/>
+      <c r="H113" s="2" t="inlineStr"/>
+    </row>
+    <row r="114" ht="28" customHeight="1">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-113</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>Fix Mark Resolved sans session active</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>Corrige _doWorkOrderClose : appelle saveActiveInterventionSession avant closeActiveInterventionSession pour garantir qu'une session est créée et que diagnosis/action_taken/outcome sont persistés, même si aucune session n'existait préalablement.</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr"/>
+      <c r="G114" s="2" t="inlineStr"/>
+      <c r="H114" s="2" t="inlineStr"/>
+    </row>
+    <row r="115" ht="28" customHeight="1">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-114</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>Rapport intervention PDF : header/footer + regroupement documents</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>Retrait Parts Replaced du PDF final, n° incident en pied de page (INC-xxx sur chaque page), documents d'intervention groupés par incident avec ExpansionTile sur la fiche équipement</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="E115" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr"/>
+      <c r="G115" s="2" t="inlineStr"/>
+      <c r="H115" s="2" t="inlineStr"/>
+    </row>
+    <row r="116" ht="28" customHeight="1">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-115</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>Clôture intervention → Disposed</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>Bouton irréparable dans TechnicianInterventionUpdateScreen : PATCH /issues/:id/close-as-disposed, issue Completed + équipement Disposed en transaction</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="E116" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr"/>
+      <c r="G116" s="2" t="inlineStr"/>
+      <c r="H116" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(issue): add related issues section and enhance issue detail screen feat(localization): update English and French translations for issue details feat(navigation): add technician module access in home hub screen test(issue): implement tests for related issues functionality chore: update verification spreadsheet
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H116"/>
+  <dimension ref="A1:H118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4188,6 +4188,66 @@
       <c r="G116" s="2" t="inlineStr"/>
       <c r="H116" s="2" t="inlineStr"/>
     </row>
+    <row r="117" ht="28" customHeight="1">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-116</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>Enrichissement fiche incident</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>Affichage localisation complète (location_text/tag), indicateur téléphone absent, section 3 incidents récents liés à l'équipement avec lien fiche équipement</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="E117" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr"/>
+      <c r="G117" s="2" t="inlineStr"/>
+      <c r="H117" s="2" t="inlineStr"/>
+    </row>
+    <row r="118" ht="28" customHeight="1">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-117</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>Fix nav hub technicien mobile</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>Ajout bouton CTA permanent + badge dans le hub technicien pour accéder à TechnicianUpdateScreen depuis le hub mobile. Refactoring _buildPmTile/_buildIssueTile avec onTap paramètre.</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="E118" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr"/>
+      <c r="G118" s="2" t="inlineStr"/>
+      <c r="H118" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add intervention documents tab for technicians
- Implemented a new tab for viewing intervention documents in the technician update screen.
- Added localization support for English and French.
- Created API endpoints for fetching intervention documents and technicians.
- Introduced filtering options by technician and date range.
- Enabled downloading documents as ZIP and printing as PDF.
- Updated user roles to include permission for viewing intervention documents.
- Enhanced the EquipmentDocument model to include additional fields.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H118"/>
+  <dimension ref="A1:H119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4248,6 +4248,36 @@
       <c r="G118" s="2" t="inlineStr"/>
       <c r="H118" s="2" t="inlineStr"/>
     </row>
+    <row r="119" ht="28" customHeight="1">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-118</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>Onglet Documents interventions (page technicien)</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>Liste/filtre par technicien et periode des documents d'intervention cross-equipement, export ZIP et impression PDF fusionnee, nouvelle permission viewInterventionDocuments</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="E119" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="inlineStr"/>
+      <c r="G119" s="2" t="inlineStr"/>
+      <c r="H119" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(push-notifications): enhance push notification banner with iOS installation guide and support messages
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H119"/>
+  <dimension ref="A1:H120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4278,6 +4278,36 @@
       <c r="G119" s="2" t="inlineStr"/>
       <c r="H119" s="2" t="inlineStr"/>
     </row>
+    <row r="120" ht="28" customHeight="1">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-119</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>Guide installation PWA iOS pour notifications</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>Détection iOS/standalone/support Push/permission refusée, guidant l'ajout à l'écran d'accueil requis par Safari pour les notifications push app fermée</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="E120" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr"/>
+      <c r="G120" s="2" t="inlineStr"/>
+      <c r="H120" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add final equipment report API and PDF generation
- Implemented GET /api/equipment/:id/final-report to return a consolidated summary and history of resolved interventions for equipment.
- Added logic to calculate KPIs such as MTTR, reopened rate, and total downtime.
- Created a new utility for building the final report data structure.
- Developed PDF generation for the final equipment report, including a summary of KPIs and a detailed intervention history.
- Updated document types to include 'final_report'.
- Enhanced the technician intervention update screen to allow inline document uploads.
- Added tests for the final report API to ensure correct functionality and data integrity.
- Updated localization files for new UI elements related to document uploads.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H120"/>
+  <dimension ref="A1:H121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4308,6 +4308,36 @@
       <c r="G120" s="2" t="inlineStr"/>
       <c r="H120" s="2" t="inlineStr"/>
     </row>
+    <row r="121" ht="28" customHeight="1">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-120</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>Case document inline + rapport final équipement</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>Case a cocher inline remplace le dialog post-hoc d'ajout de document ; generation auto d'un rapport final equipement (resume interventions + KPI MTTR/reouverture/downtime) a chaque Mark Resolved</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="E121" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="inlineStr"/>
+      <c r="G121" s="2" t="inlineStr"/>
+      <c r="H121" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(intervention-documents): enhance document filtering by type and update UI components
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H121"/>
+  <dimension ref="A1:H122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4338,6 +4338,36 @@
       <c r="G121" s="2" t="inlineStr"/>
       <c r="H121" s="2" t="inlineStr"/>
     </row>
+    <row r="122" ht="28" customHeight="1">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-121</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>Filtre type document intervention</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>Cases a cocher (rapport d'intervention / rapport de fin d'intervention) pour filtrer liste + export ZIP/PDF de l'onglet Documents technicien</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="E122" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr"/>
+      <c r="G122" s="2" t="inlineStr"/>
+      <c r="H122" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Enhance user management and incident handling
- Added userId to _RoleRequest model for better role request tracking.
- Implemented user detail navigation from role requests in UserManagementScreen.
- Introduced CountBadge widget for displaying notification and sidebar item counts.
- Refactored EquipmentIncidentsTab to use _IssueCard for better state management and UI.
- Removed deprecated issue validation sheet widget to streamline codebase.
- Updated AppSidebar and NotificationBell to utilize CountBadge for improved notification display.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H122"/>
+  <dimension ref="A1:H126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4368,6 +4368,134 @@
       <c r="G122" s="2" t="inlineStr"/>
       <c r="H122" s="2" t="inlineStr"/>
     </row>
+    <row r="123" ht="28" customHeight="1">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-122</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>Navigation demande de rôle vers détail utilisateur</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>Ligne de demande de rôle cliquable vers UserDetailScreen ; validation/rejet possible depuis l'écran de détail (même logique que les demandes de département)</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="E123" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="inlineStr"/>
+      <c r="G123" s="2" t="inlineStr"/>
+      <c r="H123" s="2" t="inlineStr"/>
+    </row>
+    <row r="124" ht="28" customHeight="1">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-123</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>Badge validation + scission par groupe technicien</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>Badge rouge sidebar (compteur incidents a valider par groupe) et separation de l'onglet A valider en 2 listes (mon groupe validable / autres techniciens lecture seule)</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="E124" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr"/>
+      <c r="G124" s="2" t="inlineStr"/>
+      <c r="H124" s="2" t="inlineStr"/>
+    </row>
+    <row r="125" ht="28" customHeight="1">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-124</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>Détails intervention + documents dans onglet Incidents</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>Panneau dépliable par incident (diagnostic, actions, durée, coût, documents PDF) dans l'onglet Incidents de la fiche équipement, sans changement backend</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="E125" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr"/>
+      <c r="G125" s="2" t="inlineStr"/>
+      <c r="H125" s="2" t="inlineStr">
+        <is>
+          <t>flutter analyze OK (0 erreur). Test manuel navigateur non effectué (Keycloak/auth-service indisponibles en local, décision utilisateur de skip). Refactor /simplify : carte incident extraite en StatefulWidget dédié (état d'expansion local par carte au lieu d'un Set au niveau de l'onglet), formatage coût aligné sur le format existant (toStringAsFixed(0) + RWF).</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="28" customHeight="1">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-125</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>Fiche détail incident + rejet technicien</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>Navigation carte 'À valider' vers la fiche détail incident avec bandeau Valider/Rejeter, correctif RBAC permettant aux techniciens de rejeter, document PDF de rejet archivé sur l'équipement</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="E126" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr"/>
+      <c r="G126" s="2" t="inlineStr"/>
+      <c r="H126" s="2" t="inlineStr">
+        <is>
+          <t>flutter analyze 0 erreur, npm test db-service 281/281 passés. Vérification manuelle non effectuée (stack Keycloak indisponible dans cet environnement).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add final intervention report generation and attachment handling
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H126"/>
+  <dimension ref="A1:H127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4496,6 +4496,36 @@
         </is>
       </c>
     </row>
+    <row r="127" ht="28" customHeight="1">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-126</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>Annexes rapport intervention + rapport final par incident</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>Section annexes indexée (documents/photos) sur le rapport d'intervention ; nouveau rapport final par incident (KPI + résumé) généré systématiquement au Mark Resolved, y compris sans équipement lié</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="E127" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F127" s="2" t="inlineStr"/>
+      <c r="G127" s="2" t="inlineStr"/>
+      <c r="H127" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add issue_id filter for PDF merging in intervention documents
- Introduced optional `issue_id` parameter for the `/print-pdf` endpoint to allow merging of PDFs for a specific incident.
- Updated SQL query parsing to include `issue_id` in filter validation.
- Enhanced document retrieval logic to support grouping by `issue_id`.
- Implemented new utility functions for grouping and formatting intervention documents.
- Added tests to verify functionality of the new `issue_id` filter and document grouping.
- Updated localization files for new messages related to PDF merging.
- Refactored UI components to utilize the new document grouping logic.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H127"/>
+  <dimension ref="A1:H129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4526,6 +4526,66 @@
       <c r="G127" s="2" t="inlineStr"/>
       <c r="H127" s="2" t="inlineStr"/>
     </row>
+    <row r="128" ht="28" customHeight="1">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-127</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>Fermeture auto fiche incident après validation</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>IssueDetailScreen se ferme automatiquement après Valider/Rejeter réussi (Navigator.pop), alignée sur le pattern equipment_detail_screen.dart:583-587</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="E128" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr"/>
+      <c r="G128" s="2" t="inlineStr"/>
+      <c r="H128" s="2" t="inlineStr"/>
+    </row>
+    <row r="129" ht="28" customHeight="1">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-128</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>Regroupement par issue + export PDF fusionné (onglet Documents technicien)</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>Documents d'intervention groupés par issue (ExpansionTile, tri par date d'incident) sur l'onglet technicien cross-équipement, avec bouton de fusion PDF par groupe (endpoint /print-pdf étendu avec issue_id).</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="E129" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F129" s="2" t="inlineStr"/>
+      <c r="G129" s="2" t="inlineStr"/>
+      <c r="H129" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Enhance intervention document handling with annex support
- Implemented text extraction from PDF content streams using zlib.
- Added functionality to create and manage annex numbers for completion documents.
- Updated the database schema to include annex_number and annex_type_index for documents.
- Enhanced the API to support merging intervention documents with annexes, including proper pagination and ordering.
- Improved localization for intervention and annex sections in the Flutter app.
- Refactored document grouping logic to separate intervention and annex documents, ensuring correct sorting by annex number.
- Added tests to verify the new functionality and ensure proper document handling.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H129"/>
+  <dimension ref="A1:H130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4586,6 +4586,40 @@
       <c r="G129" s="2" t="inlineStr"/>
       <c r="H129" s="2" t="inlineStr"/>
     </row>
+    <row r="130" ht="28" customHeight="1">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-129</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>Sous-groupes Intervention/Annexe + tampon PDF + sommaire</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>Onglet Documents technicien : sous-sections Intervention/Annexe par incident, tampon PDF permanent (annexe N, incident, page) sur pièces jointes et photos dès l'upload, sommaire conditionnel et réordonnancement du merge PDF par incident (rapport final -&gt; sommaire -&gt; intervention -&gt; annexes).</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="E130" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr"/>
+      <c r="G130" s="2" t="inlineStr"/>
+      <c r="H130" s="2" t="inlineStr">
+        <is>
+          <t>Backend : 296 tests db-service passent (dont annex_stamp_service.test.js, intervention_documents.test.js). Flutter : flutter analyze --no-fatal-infos 0 erreur. Vérification navigateur non effectuée (stack Keycloak/Docker indisponible dans cet environnement).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Enhance intervention documents handling with photo support
- Added support for 'photo' document type in intervention documents routes.
- Updated filtering logic to include/exclude photos based on user input.
- Modified database queries to handle photo documents alongside intervention and completion documents.
- Updated PDF generation to include photos when requested.
- Enhanced ZIP export functionality to include photos.
- Updated localization files to reflect new document types and counts in UI.
- Added tests to ensure correct behavior for new photo handling in various scenarios.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H130"/>
+  <dimension ref="A1:H131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4620,6 +4620,36 @@
         </is>
       </c>
     </row>
+    <row r="131" ht="28" customHeight="1">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-130</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>Cases à cocher export documents technicien</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>3 cases (Intervention/Piece jointe/Photo) pilotant liste + exports ZIP/PDF (global et par incident), rapport final toujours inclus, onglet scrollable mobile</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="E131" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="inlineStr"/>
+      <c r="G131" s="2" t="inlineStr"/>
+      <c r="H131" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Enhance issue form buttons and layout; add installation guide link in login screen; implement offline detection and fallback; update manifest for PWA; create installation page and poster; improve SSL certificate handling in setup script; update verification spreadsheet
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H133"/>
+  <dimension ref="A1:H136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4718,6 +4718,108 @@
         </is>
       </c>
     </row>
+    <row r="134" ht="28" customHeight="1">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-133</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>Onglets page détail incident</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>Réorganisation de IssueDetailScreen en 4 onglets (Identification/Intervention/Documents/Historique), onglet Documents masqué pour hospitalStaff</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="E134" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr"/>
+      <c r="G134" s="2" t="inlineStr"/>
+      <c r="H134" s="2" t="inlineStr">
+        <is>
+          <t>flutter analyze OK (0 erreur sur le fichier). Test manuel navigateur non effectué (stack Keycloak+backend indisponible en sandbox) - à valider manuellement avant mise en prod.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="28" customHeight="1">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-134</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>Fix boutons rognés étape 2 signalement mobile</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>Row 3 boutons Retour/Annuler/Envoyer remplacée par Column 2 lignes (Retour+Annuler / Envoyer pleine largeur) + hauteur tactile min 48dp, corrige le rognage du bouton Annuler sur téléphone</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="E135" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F135" s="2" t="inlineStr"/>
+      <c r="G135" s="2" t="inlineStr"/>
+      <c r="H135" s="2" t="inlineStr">
+        <is>
+          <t>flutter analyze OK (0 erreur sur le fichier). Vérification navigateur impossible dans cet environnement (bug preexistant: chemin avec espaces casse le hook de build native assets objective_c pour flutter run).</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="28" customHeight="1">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-135</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>PWA installable + CA interne + page offline</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>CA interne 2 étages avec page /setup/ guidée (Android/iOS/PC + QR), page offline anglaise via SW, fusion SW dans build_and_push.sh, mise à jour silencieuse vérifiée</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="E136" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr"/>
+      <c r="G136" s="2" t="inlineStr"/>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t>Renouvellement cert sans action téléphone ; saisie offline volontairement hors scope ; SW Flutter 3.41 = stub sans cache, précache offline.html assuré par push_sw.js</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Remove update button from issue detail screens and localization files
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H136"/>
+  <dimension ref="A1:H137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4820,6 +4820,40 @@
         </is>
       </c>
     </row>
+    <row r="137" ht="28" customHeight="1">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-136</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>Suppression bouton Mettre a jour l'incident</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>Retrait du bouton redondant en bas de la page detail incident (IssueDetailScreen) qui dupliquait l'onglet Intervention ; nettoyage du callback onNavigate devenu mort et de la cle i18n associee.</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="E137" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="inlineStr"/>
+      <c r="G137" s="2" t="inlineStr"/>
+      <c r="H137" s="2" t="inlineStr">
+        <is>
+          <t>flutter analyze --no-fatal-infos OK sur issue_detail_screen.dart et issue_tracking_screen.dart</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor intervention tracking and follow-up features
- Updated English and French localization strings for intervention and follow-up sections.
- Introduced new follow-up card widget to display intervention session details.
- Enhanced issue intervention session model to include next action due date.
- Modified issue detail screen to integrate the new follow-up card.
- Added functionality for selecting due dates for next actions in technician intervention update screen.
- Improved document handling in intervention documents section to support new grouping logic.
- Updated document download logic to handle photos and intervention documents appropriately.
- Refactored code for better readability and maintainability.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H137"/>
+  <dimension ref="A1:H138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4854,6 +4854,40 @@
         </is>
       </c>
     </row>
+    <row r="138" ht="28" customHeight="1">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-137</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>Refonte Documents/Intervention fiche incident</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>Permission gating onglet Documents, archivage PDF dernière boucle, résumé Follow up basé sur les boucles, sous-catégorie Annexe (pièces jointes + photos) sur incident et équipement</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="E138" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr"/>
+      <c r="G138" s="2" t="inlineStr"/>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>Ajout colonne next_action_due_at ; correctif bonus splitInterventionAnnexe (photos manquantes sur onglet Documents technicien existant)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Enhance attachment upload handling and add user feedback for failures
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H138"/>
+  <dimension ref="A1:H139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4888,6 +4888,40 @@
         </is>
       </c>
     </row>
+    <row r="139" ht="28" customHeight="1">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-138</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>Corrections documents fiche incident</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>Fix glyphe cassé PDF (tiret cadratin), renommage anglais des fichiers PDF archivés, correction/surfaçage de la disparition de pièces jointes photo à la clôture Bon de Travail, audit trail des échecs de tamponnage</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="E139" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F139" s="2" t="inlineStr"/>
+      <c r="G139" s="2" t="inlineStr"/>
+      <c r="H139" s="2" t="inlineStr">
+        <is>
+          <t>Cause confirmee par inspection de code : catch(_) muet dans _uploadPickedDocumentsIfAny avalait silencieusement tout echec de POST /documents (reseau, timeout, 401 non rafraichissable, 500) sans jamais avertir le technicien ni tracer l'echec cote serveur - corrige en surfacant le resultat (retour bool + SnackBar + logAction annex_stamp_failed). Piste JPEG progressif explicitement ecartee (revertDocumentAnnexStamp garde le document en base, juste sans annex_number) mais en ecrivant le test de non-regression demande, un VRAI bug a ete trouve et corrige dans annex_stamp_service.js : JpegEmbedder de pdf-lib lit imageData.buffer sans respecter byteOffset/byteLength, ce qui casse sur tout buffer issu du pool interne de Node (fichiers &lt; 4 Ko lus via fs.readFileSync) meme si le JPEG source est valide - corrige par une recopie defensive dans un buffer non poole avant embedJpg/embedPng, avec test de regression dedie. Piste ordre des operations (upload apres plusieurs awaits non catches dans _doWorkOrderClose) confirmee comme risque residuel documente, non modifiee (hors perimetre du prompt). Verification : npm test db-service 315/315 OK, flutter analyze 0 erreur. Docker indisponible dans cet environnement -&gt; scenarios manuels UI non rejoues en direct, valides par inspection de code + tests automatises cibles.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Implement photo grid PDF generation for intervention documents and enhance error handling
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H139"/>
+  <dimension ref="A1:H140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4922,6 +4922,40 @@
         </is>
       </c>
     </row>
+    <row r="140" ht="28" customHeight="1">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-139</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>Correctifs documents intervention &amp; fusion PDF</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>Reordonnancement upload pieces jointes avant generation rapport final, logging erreurs fusion PDF, grille 2x2 photos annexees</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="E140" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr"/>
+      <c r="G140" s="2" t="inlineStr"/>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>4 correctifs, aucun changement de schema DB</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Update issue form localization keys and enhance equipment search handling
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H140"/>
+  <dimension ref="A1:H141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4956,6 +4956,40 @@
         </is>
       </c>
     </row>
+    <row r="141" ht="28" customHeight="1">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-140</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>Uniformisation champ équipement signalement</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>Champ Related Equipment (recherche par tag number, cross-catégorie) uniformisé sur les 4 onglets Bio/Infra/IT/Autre du formulaire de signalement d'incident</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="E141" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr"/>
+      <c r="G141" s="2" t="inlineStr"/>
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t>EquipmentPickerField conservé (encore utilisé dans issue_detail_screen.dart, contrairement à l'hypothèse initiale) ; flutter analyze OK ; /simplify appliqué (4 agents en parallèle)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Implement soft delete for intervention documents and enhance upload error handling
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H141"/>
+  <dimension ref="A1:H144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4990,6 +4990,104 @@
         </is>
       </c>
     </row>
+    <row r="142" ht="28" customHeight="1">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-141</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>Upload immédiat pièces jointes intervention</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>Corrige la lenteur de Save-and-Close (upload décalé à la sélection du fichier) et l'absence de documents dans l'onglet Documents (fix TypeError _parseMultipartResponse + stream reload). Ajout DELETE /api/issues/:id/documents/:doc_id avec contrôle d'auteur.</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="E142" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr"/>
+      <c r="G142" s="2" t="inlineStr"/>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>Cas A: tamponnage synchrone dans la réponse HTTP, upload déclenché maintenant à la sélection. Cas B: bug de cast JSON (Array vs Map) + état figé de InterventionDocumentsTab — corrigé via _PendingUpload + StreamController&lt;void&gt; broadcast.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="28" customHeight="1">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-142</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>Autocomplétion équipement IssueForm</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>Remplace champ tag + bouton recherche par RawAutocomplete&lt;Equipment&gt; sur les 4 onglets, recherche locale nom+tags, compatible QR scan et hasUnsavedData</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="E143" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr"/>
+      <c r="G143" s="2" t="inlineStr"/>
+      <c r="H143" s="2" t="inlineStr"/>
+    </row>
+    <row r="144" ht="28" customHeight="1">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-143</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>Raison affichée pour échec upload pièce jointe intervention</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>Le message de clôture 'Closed successfully, but some files could not be uploaded' n'affichait que les noms de fichiers sans expliquer pourquoi. Capture désormais le message d'erreur serveur (type non supporté, fichier trop volumineux, etc.) et l'affiche dans le SnackBar de clôture + tooltip sur le chip du fichier en échec.</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="E144" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr"/>
+      <c r="G144" s="2" t="inlineStr"/>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>Fichier: technician_intervention_update_screen.dart. Le serveur renvoyait déjà un message JSON exploitable (index.js:86-98), il était juste ignoré côté client (catch (e) -&gt; debugPrint seul).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add uploader tracking to incident photos and enhance document download naming
- Added `uploaded_by` and `uploader_name` columns to `issue_photos` table for tracking the uploader's identity.
- Updated document download functionality to generate a friendly filename that includes equipment name, tag number, issue ID, and annex number.
- Enhanced the `sendStoredDocument` function to accept an optional friendly name for downloads.
- Modified various routes to include the new uploader information and friendly naming in responses and downloads.
- Updated Flutter models and screens to accommodate the new `equipmentTag` and uploader details for better display and reporting.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H144"/>
+  <dimension ref="A1:H145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5088,6 +5088,36 @@
         </is>
       </c>
     </row>
+    <row r="145" ht="28" customHeight="1">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-144</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>Correctifs annexes intervention</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>Uploader photos issue tracé (uploaded_by/uploader_name), tag_number equipement affiche dans les rapports PDF (loop/final), nom de telechargement convivial (equipement-tag-issue-annexe) pour photos/documents et export ZIP.</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="E145" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr"/>
+      <c r="G145" s="2" t="inlineStr"/>
+      <c r="H145" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add monthly report job tests and adjust RBAC for supervisor role
- Implemented tests for the monthly report job, ensuring correct KPI calculations and report sending.
- Updated RBAC rules to restrict supervisor role from modifying incidents while retaining access to reporting functionalities.
- Enhanced notification preferences to include monthly report settings for supervisors and admins.
- Adjusted user role permissions to reflect the new responsibilities of the supervisor role.
- Modified Docker Compose configurations to improve security and compatibility with snap installations.
- Updated setup script to handle password inputs more securely.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H145"/>
+  <dimension ref="A1:H151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5118,6 +5118,206 @@
       <c r="G145" s="2" t="inlineStr"/>
       <c r="H145" s="2" t="inlineStr"/>
     </row>
+    <row r="146" ht="28" customHeight="1">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-145</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>Instrumentation KPI des skills + /improve-skill</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>Base SQLite hors repo (~/.claude/skills-data) + contexte vivant par skill + script skill_metrics.py (durée/tokens/qualité). /feature-to-prompt instrumenté (phases 0-pré et 7), nouveau skill /improve-skill (analyse KPI + amélioration SKILL.md).</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="E146" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr"/>
+      <c r="G146" s="2" t="inlineStr"/>
+      <c r="H146" s="2" t="inlineStr">
+        <is>
+          <t>Contrat commun : .claude/skills/_shared/INSTRUMENTATION.md. Script testé (start/end/report/log-improvement, mesure tokens réelle).</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="28" customHeight="1">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-146</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>Boucle KPI des prompts générés (feature-prompt-exec)</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>Les prompts produits par /feature-to-prompt embarquent 2 sections obligatoires : Suivi KPI de l'exécution (run feature-prompt-exec + label slug, affichage KPI fin d'implémentation) et Amélioration continue (/improve-skill mode retour d'exécution vers feature-to-prompt).</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="E147" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F147" s="2" t="inlineStr"/>
+      <c r="G147" s="2" t="inlineStr"/>
+      <c r="H147" s="2" t="inlineStr">
+        <is>
+          <t>skill_metrics.py : colonne label (migration idempotente) + --label sur start. improve-skill : Phase R (modif SKILL.md seulement si défaut récurrent &gt;= 2 exécutions).</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="28" customHeight="1">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-147</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>Mémoire de recherche + matrice modèles/efforts des skills</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>feature-to-prompt : RESEARCH.md hors repo (cache comparaisons marché, ancrages code, refs) consulté avant toute recherche ; PARAMS.json hors repo (exécuteur/modèle/effort par phase, subagents haiku/opus). improve-skill : 3 leviers (SKILL.md, PARAMS.json 1 param à la fois avec corrélation params v&lt;N&gt;-KPIs, consolidation RESEARCH.md) + auto-réglage de sa propre matrice.</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="E148" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr"/>
+      <c r="G148" s="2" t="inlineStr"/>
+      <c r="H148" s="2" t="inlineStr">
+        <is>
+          <t>Défauts versionnés : params.default.json + research.template.md dans chaque dossier de skill. Contrat mis à jour dans _shared/INSTRUMENTATION.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="28" customHeight="1">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-148</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>Benchmark web des skills + 5 améliorations</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>Recherche web sur les skills comparables (claude-improve, claude-reflect, prompt-architect, sdd-brainstorm, superpowers, skill-creator Anthropic), archivée dans les RESEARCH.md hors repo. Appliqué : snapshot/rollback versions/ + confiance/décroissance des leçons (improve-skill) ; score v0 + arbre par type de feature + 2-3 options d'approche (feature-to-prompt).</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="E149" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F149" s="2" t="inlineStr"/>
+      <c r="G149" s="2" t="inlineStr"/>
+      <c r="H149" s="2" t="inlineStr">
+        <is>
+          <t>Suivi d'acceptation écarté par l'utilisateur. Pistes non retenues (éval train/test, OTel) notées dans RESEARCH.md improve-skill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="28" customHeight="1">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-149</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>Rôle supervisor consultation+rapports</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>Retrait approveRequests/assignTasks, ajout generateReports, 403 backend mutations issues, ordre sidebar, rapport KPI mensuel par email (cron + Brevo + opt-out)</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="E150" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr"/>
+      <c r="G150" s="2" t="inlineStr"/>
+      <c r="H150" s="2" t="inlineStr">
+        <is>
+          <t>Migration one-shot _supervisor_role_v2; cron 0 6 1 * *; route debug send-monthly-report; toggle opt-out Flutter; analytics ajouté au module équipement</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="28" customHeight="1">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-150</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>Auto-réparation verifyEmail realm Keycloak</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>auth-service détecte et corrige au démarrage toute dérive du réglage realm verifyEmail (doit rester false), qui bloquait le login des nouveaux comptes access-request quand le script de déploiement Jenkins échouait silencieusement (|| true)</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="E151" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F151" s="2" t="inlineStr"/>
+      <c r="G151" s="2" t="inlineStr"/>
+      <c r="H151" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(equipment): implement CSV import functionality with role-based access control
- Added unit tests for CSV import functionality, covering role-based access and validation scenarios.
- Enhanced localization files for English and French to support new CSV import features.
- Updated the Equipment model to include createdById and createdByName fields.
- Implemented UI components for CSV import in the equipment form and list screens.
- Added methods in DbApiService for handling CSV file uploads and processing.
- Included error handling and reporting for CSV import operations.
- Introduced a download template feature for CSV imports.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H151"/>
+  <dimension ref="A1:H152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5318,6 +5318,36 @@
       <c r="G151" s="2" t="inlineStr"/>
       <c r="H151" s="2" t="inlineStr"/>
     </row>
+    <row r="152" ht="28" customHeight="1">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-151</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>Import CSV équipements + correctif formulaire (warranty_end_date)</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>Route POST /api/equipment/import-csv (RBAC admin/supervisor/technicien*, dry-run, slug anti-collision, doublon serial_number), colonnes created_by_id/name, champ warranty_end_date ajouté au formulaire Nouvel équipement, UI Flutter (bouton+dialog+modèle CSV+rapport erreurs).</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="E152" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F152" s="2" t="inlineStr"/>
+      <c r="G152" s="2" t="inlineStr"/>
+      <c r="H152" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(localization): update French translations for user management and settings
- Added new French translations for user-related notifications and settings.
- Updated various screens to utilize localized strings for better internationalization support.
- Improved user feedback messages for department and role requests.
- Enhanced error handling messages with localized content.
- Updated UI elements to reflect localized labels for better user experience.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H152"/>
+  <dimension ref="A1:H153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5348,6 +5348,36 @@
       <c r="G152" s="2" t="inlineStr"/>
       <c r="H152" s="2" t="inlineStr"/>
     </row>
+    <row r="153" ht="28" customHeight="1">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-152</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>Audit et correction i18n résiduel</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>Correction des chaînes françaises en dur dans écrans+widgets Flutter, rapport audit/rapport_i18n_2026-07-06.md</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="E153" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F153" s="2" t="inlineStr"/>
+      <c r="G153" s="2" t="inlineStr"/>
+      <c r="H153" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Enhance Equipment Analytics and Reporting Features
- Updated EquipmentListScreen to include additional columns for subcategory, macro-category, creation date, and creator.
- Renamed ReportsScreen to Equipment Analytics and updated navigation labels accordingly.
- Added new KPIs to the reports section, including MTBF, issue backlog, obsolescence rate, criticality breakdown, and total downtime.
- Implemented GmaoKpiSectionExtra widget to display new KPIs in a responsive grid layout.
- Updated localization files for English and French to reflect new terminology and added translations for new KPI indicators.
- Created update.sh script for automated deployment updates, including backup and service health checks.
- Modified CSV export functionality in EquipmentListScreen to include new fields.
- Updated verification spreadsheet to reflect changes in reporting and analytics.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H153"/>
+  <dimension ref="A1:H156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5378,6 +5378,100 @@
       <c r="G153" s="2" t="inlineStr"/>
       <c r="H153" s="2" t="inlineStr"/>
     </row>
+    <row r="154" ht="28" customHeight="1">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-153</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>Script update.sh</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>Mise à jour d'un déploiement IP-only déjà provisionné (backup auto + pull + restart + re-sync rôles Keycloak)</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="E154" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr"/>
+      <c r="G154" s="2" t="inlineStr"/>
+      <c r="H154" s="2" t="inlineStr"/>
+    </row>
+    <row r="155" ht="28" customHeight="1">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-154</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>Fix seed Keycloak non-idempotent (Jenkins)</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>keycloak-seed.js recréait les comptes démo supprimés à chaque déploiement Jenkins (prod+dev) car il ne vérifiait que l'existence par email, pas l'historique de suppression. Ajout d'un attribut realm demoSeeded, vérifié avant tout seed.</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="E155" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F155" s="2" t="inlineStr"/>
+      <c r="G155" s="2" t="inlineStr"/>
+      <c r="H155" s="2" t="inlineStr">
+        <is>
+          <t>auth-service/scripts/keycloak-seed.js modifié. Jenkinsfile inchangé (fix contenu dans le script). npm test auth-service : 206/206 OK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="28" customHeight="1">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-155</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>Analytics Équipements + KPI + export CSV enrichi</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>Renommage ReportsScreen en Analytics Équipements, ajout MTBF/backlog/obsolescence/criticité ABC/downtime, 4 colonnes CSV supplémentaires</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="E156" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr"/>
+      <c r="G156" s="2" t="inlineStr"/>
+      <c r="H156" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix navigation labels and update PDF report service documentation
- Updated the navigation label for 'reports' to 'analytics' in role_detail_screen.dart.
- Corrected the documentation comment in pdf_report_service.dart to reflect that data is passed from ReportsTab instead of ReportsScreen.
- Updated the verification Excel file to reflect recent changes.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H156"/>
+  <dimension ref="A1:H157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5472,6 +5472,36 @@
       <c r="G156" s="2" t="inlineStr"/>
       <c r="H156" s="2" t="inlineStr"/>
     </row>
+    <row r="157" ht="28" customHeight="1">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-156</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>Fusion Reports+Analytics</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr">
+        <is>
+          <t>Ecrans ReportsScreen et AnalyticsScreen fusionnes en un seul ecran Analytics a 2 onglets (Rapports / Analytique)</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="E157" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F157" s="2" t="inlineStr"/>
+      <c r="G157" s="2" t="inlineStr"/>
+      <c r="H157" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(equipment): enforce unique physical tag requirement and add validation for tag usage
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H157"/>
+  <dimension ref="A1:H159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5502,6 +5502,70 @@
       <c r="G157" s="2" t="inlineStr"/>
       <c r="H157" s="2" t="inlineStr"/>
     </row>
+    <row r="158" ht="28" customHeight="1">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-157</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>Création équipement ouverte aux techniciens</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>Le bouton 'Nouvel équipement' (equipment_list_screen.dart) et la route POST /api/equipment (backend) étaient réservés à admin/supervisor ; alignés sur le garde-fou déjà utilisé pour l'import CSV (_canEdit / TECH_ROLES), ouvrant la création manuelle aux 3 rôles techniciens.</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="E158" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F158" s="2" t="inlineStr"/>
+      <c r="G158" s="2" t="inlineStr"/>
+      <c r="H158" s="2" t="inlineStr">
+        <is>
+          <t>Tests RBAC mis à jour (rbac_equipment_issues.test.js, equipment_import_csv.test.js) ; npm test (396/396) et flutter analyze OK, aucune erreur bloquante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="28" customHeight="1">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-158</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>Tag physique obligatoire</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>Tag obligatoire + unique a la creation/edition d'equipement (UI + API), unicite seule sur import CSV</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="E159" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F159" s="2" t="inlineStr"/>
+      <c r="G159" s="2" t="inlineStr"/>
+      <c r="H159" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(api): implement proactive token refresh mechanism and add tests for expiry decoding feat(localization): add 'My problem isn't in the list' message for issue form feat(issue_form): add button for 'Other' infrastructure category selection
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H159"/>
+  <dimension ref="A1:H161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5566,6 +5566,74 @@
       <c r="G159" s="2" t="inlineStr"/>
       <c r="H159" s="2" t="inlineStr"/>
     </row>
+    <row r="160" ht="28" customHeight="1">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-159</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>Raccourci Autre recherche infra</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>Bouton texte avant la recherche rapide de l'onglet Infrastructure, fixe directement _infraCategory='Other'</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="E160" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F160" s="2" t="inlineStr"/>
+      <c r="G160" s="2" t="inlineStr"/>
+      <c r="H160" s="2" t="inlineStr">
+        <is>
+          <t>UI only, aucun changement backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="28" customHeight="1">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-160</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>Fix déconnexions - race condition refresh token</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>Verrou de concurrence sur ApiClient._tryRefresh (rotation stricte Keycloak), refresh proactif avant expiration, idempotence des durées de session dans keycloak-init.js</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="E161" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F161" s="2" t="inlineStr"/>
+      <c r="G161" s="2" t="inlineStr"/>
+      <c r="H161" s="2" t="inlineStr">
+        <is>
+          <t>flutter analyze vert (0 erreur) ; npm test auth-service 206/206 vert ; flutter test bloqué par bug environnement pré-existant (hook natif objective_c casse sur espace du chemin projet, indépendant du fix) ; vérification manuelle par trace de code (stack Keycloak/Docker non démarré) ; hypothèse PUT partiel Keycloak différée (Docker indisponible)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update French localization strings for improved clarity and accuracy
- Corrected translations for navigation items, issue reporting, and common terms.
- Enhanced descriptions for issue categories and forms to better reflect their purpose.
- Adjusted urgency labels and reporting terminology for consistency across the application.
- Updated the English localization to match the changes made in French.
- Modified the verification spreadsheet to reflect the latest updates.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H161"/>
+  <dimension ref="A1:H162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5634,6 +5634,40 @@
         </is>
       </c>
     </row>
+    <row r="162" ht="28" customHeight="1">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-161</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>Audit UX parcours incident</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>Audit multi-agents oeil neuf du parcours de signalement (5 segments, FR+EN) : rapport, correctifs ARB, prompts par page</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="E162" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr"/>
+      <c r="G162" s="2" t="inlineStr"/>
+      <c r="H162" s="2" t="inlineStr">
+        <is>
+          <t>50 constats (0 bloquant, 20 genants, 30 mineurs), 0 refute ; 24 couverts par ARB ; 4 prompts pages 1/3/4/5 ; passe navigateur en repli statique (Docker indisponible)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(issue-form): enhance user guidance with detailed hints and urgency information
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H162"/>
+  <dimension ref="A1:H163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5668,6 +5668,36 @@
         </is>
       </c>
     </row>
+    <row r="163" ht="28" customHeight="1">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-162</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>Aide novice formulaire d'incident</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>Bandeau d'intro, hints enrichis (tag/description), rappel SLA par urgence, aide non répertorié - IssueFormScreen, 4 onglets</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="E163" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F163" s="2" t="inlineStr"/>
+      <c r="G163" s="2" t="inlineStr"/>
+      <c r="H163" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Implement equipment linking and correction functionality
- Added the ability to link equipment to issues and correct already linked equipment.
- Updated API service to handle linking with a reason for corrections.
- Created a reusable dialog for linking and correcting equipment.
- Enhanced tests for linking equipment, including validation for reasons.
- Updated localization files for new strings related to equipment linking and corrections.
- Modified screens to utilize the new equipment linking dialog.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H163"/>
+  <dimension ref="A1:H165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5698,6 +5698,66 @@
       <c r="G163" s="2" t="inlineStr"/>
       <c r="H163" s="2" t="inlineStr"/>
     </row>
+    <row r="164" ht="28" customHeight="1">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-163</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>Correction équipement lié à un incident</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>PATCH /link-equipment débloqué pour corriger un équipement déjà lié (motif obligatoire), UI ajoutée sur IssueDetailScreen et TechnicianInterventionUpdateScreen</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="E164" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr"/>
+      <c r="G164" s="2" t="inlineStr"/>
+      <c r="H164" s="2" t="inlineStr"/>
+    </row>
+    <row r="165" ht="28" customHeight="1">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-164</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>Logs de diffusion notifications + test broadcast</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>Journalisation agrégée de send-to-roles (table logs) + bouton de test multi-rôles dans la page Debug, historique persisté</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="E165" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F165" s="2" t="inlineStr"/>
+      <c r="G165" s="2" t="inlineStr"/>
+      <c r="H165" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor(issue-form): remove urgency help text and improve scrolling behavior
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H165"/>
+  <dimension ref="A1:H166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5758,6 +5758,36 @@
       <c r="G165" s="2" t="inlineStr"/>
       <c r="H165" s="2" t="inlineStr"/>
     </row>
+    <row r="166" ht="28" customHeight="1">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-165</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>Fix upload photos + UX formulaire signalement</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>Correction du parsing de réponse multipart (faux échec + duplication au retry dans le cas nominal), suppression du texte SLA sous l'urgence, reset du scroll au changement d'étape</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="E166" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr"/>
+      <c r="G166" s="2" t="inlineStr"/>
+      <c r="H166" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Implement PM Protocol Management Screen
- Added PmProtocolsScreen for managing PM protocols associated with equipment subcategories.
- Integrated CRUD operations for PM protocols in DbApiService.
- Created CatalogSearchField widget for searchable dropdowns with create option.
- Developed EquipmentCatalogEditDialog for editing equipment brand and model.
- Enhanced EquipmentInfoTab and EquipmentMaintenanceTab to support PM protocol management.
- Updated PmChecklistWidget to allow comments and compliance status for checklist items.
- Added error handling and loading states for better user experience.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H166"/>
+  <dimension ref="A1:H168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5788,6 +5788,74 @@
       <c r="G166" s="2" t="inlineStr"/>
       <c r="H166" s="2" t="inlineStr"/>
     </row>
+    <row r="167" ht="28" customHeight="1">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-166</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>Gestion protocoles PM depuis fiche équipement</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>CRUD protocoles PM par sous-catégorie (écrans liste/formulaire), RBAC POST/PUT élargi à supervisor+techniciens, commentaire + Pass/Fail par tâche à la validation avec auto-création d'incident consolidé, historique enrichi du checklist_snapshot</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="E167" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F167" s="2" t="inlineStr"/>
+      <c r="G167" s="2" t="inlineStr"/>
+      <c r="H167" s="2" t="inlineStr">
+        <is>
+          <t>419 tests backend + flutter analyze OK ; flutter test bloqué par limitation environnement connue (hook native asset objective_c casse sur espace du chemin, cf run #8 mémoire)</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" ht="28" customHeight="1">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-167</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>Sélecteur catalogue Fabricant/Modèle (recherche + ajout)</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>Dialog unifié recherche+dropdown+ajouter pour rattacher fabricant/modèle catalogue depuis la fiche détail équipement, remplace l'édition texte libre ; RBAC POST/PUT brands+models aligné sur PUT équipement</t>
+        </is>
+      </c>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="E168" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F168" s="2" t="inlineStr"/>
+      <c r="G168" s="2" t="inlineStr"/>
+      <c r="H168" s="2" t="inlineStr">
+        <is>
+          <t>Composant CatalogSearchField réutilisable (RawAutocomplete, zéro dépendance). Test manuel navigateur non exécuté (Docker/Keycloak non démarré dans l'environnement) — edge cases tracés contre le code à la place.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Implement push notification diagnostics and testing features
- Added endpoints for subscribing and unsubscribing to push notifications.
- Enhanced subscription management to include platform information.
- Introduced a test push notification feature for users to verify push functionality.
- Created an admin diagnostic view to list all active push subscriptions.
- Updated localization files for new push notification messages.
- Implemented structured results for push notification tests.
- Enhanced error handling and logging for push notifications.
- Updated the service worker to acknowledge receipt of push notifications.
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H168"/>
+  <dimension ref="A1:H169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5856,6 +5856,36 @@
         </is>
       </c>
     </row>
+    <row r="169" ht="28" customHeight="1">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-168</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>Diagnostic + observabilité push iOS</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>Distinction 'accepté par le service push' vs 'confirmé reçu sur l'appareil' (accusé de réception SW), bouton self-test, écran admin de diagnostic des souscriptions push.</t>
+        </is>
+      </c>
+      <c r="D169" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="E169" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F169" s="2" t="inlineStr"/>
+      <c r="G169" s="2" t="inlineStr"/>
+      <c r="H169" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor(equipment): update tag number validation logic for PUT requests
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H169"/>
+  <dimension ref="A1:H170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5886,6 +5886,40 @@
       <c r="G169" s="2" t="inlineStr"/>
       <c r="H169" s="2" t="inlineStr"/>
     </row>
+    <row r="170" ht="28" customHeight="1">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-169</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>Fix validation tag_number sur PUT equipment</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>PUT /api/equipment/:id n'exige plus tag_number sur toute edition partielle (fabricant/modele, departement, localisation...) quand l'equipement n'a pas encore de tag - seule la creation (POST) l'exige desormais, PUT valide uniquement si le champ est explicitement envoye</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="E170" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F170" s="2" t="inlineStr"/>
+      <c r="G170" s="2" t="inlineStr"/>
+      <c r="H170" s="2" t="inlineStr">
+        <is>
+          <t>Bug remonte par l'utilisateur: dialog Manufacturer/model + Save echouait avec 'Le tag physique (tag_number) est requis'. 420/420 tests db-service passent.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Add dialogs for creating new brands and models in equipment catalog
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H170"/>
+  <dimension ref="A1:H171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5920,6 +5920,36 @@
         </is>
       </c>
     </row>
+    <row r="171" ht="28" customHeight="1">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-170</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>Bouton + création fabricant/modèle</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>Bouton + explicite (dialog dédié, garde anti double-clic, message 409 spécifique) à côté des champs Fabricant/Modèle du dialog d'édition catalogue sur la fiche équipement, en complément du mécanisme de création via la recherche existante</t>
+        </is>
+      </c>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="E171" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F171" s="2" t="inlineStr"/>
+      <c r="G171" s="2" t="inlineStr"/>
+      <c r="H171" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(users): ensure email and username are retained during updates to prevent data loss
</commit_message>
<xml_diff>
--- a/verification/suivi_verifications.xlsx
+++ b/verification/suivi_verifications.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H171"/>
+  <dimension ref="A1:H172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5950,6 +5950,40 @@
       <c r="G171" s="2" t="inlineStr"/>
       <c r="H171" s="2" t="inlineStr"/>
     </row>
+    <row r="172" ht="28" customHeight="1">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-171</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>Fix compte bloque apres promotion admin</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>PUT /api/users/:id renvoyait un email/username absent quand seul le role changeait (dialogue user_detail_screen sans champ email), et Keycloak effacait l'email existant -&gt; compte injoignable au login suivant. Le endpoint renvoie desormais toujours l'email courant.</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="E172" s="3" t="inlineStr">
+        <is>
+          <t>En attente de revue</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr"/>
+      <c r="G172" s="2" t="inlineStr"/>
+      <c r="H172" s="2" t="inlineStr">
+        <is>
+          <t>auth-service/src/routes/users.js:174-186. npm test OK (206/206). A verifier en reproduisant le cas sur un compte Keycloak reel.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>